<commit_message>
updates to match description
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schirico\Repositories\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0B3E72E-1566-43C2-8877-CBC356D750BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363D2B9D-778B-46AB-A30B-0DD6DF30AD7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28920" yWindow="450" windowWidth="27705" windowHeight="15090" tabRatio="879" firstSheet="2" activeTab="12" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="9" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -530,19 +530,10 @@
     <t>MESH SIZE</t>
   </si>
   <si>
-    <t>MAX BRAIL CAPACITY</t>
-  </si>
-  <si>
     <t>MID NET STRETCHED</t>
   </si>
   <si>
     <t>BUNT STRETCHED</t>
-  </si>
-  <si>
-    <t>MAX DEPTH</t>
-  </si>
-  <si>
-    <t>MAX LENGTH</t>
   </si>
   <si>
     <t>START SETTING</t>
@@ -678,6 +669,15 @@
   </si>
   <si>
     <t>DESTINATION</t>
+  </si>
+  <si>
+    <t>MAXIMUM LENGTH</t>
+  </si>
+  <si>
+    <t>MAXIMUM DEPTH</t>
+  </si>
+  <si>
+    <t>MAXIMUM BRAIL CAPACITY</t>
   </si>
 </sst>
 </file>
@@ -1198,6 +1198,9 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1270,14 +1273,49 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1319,14 +1357,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1339,17 +1369,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1360,9 +1379,8 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1379,26 +1397,8 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1737,24 +1737,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="60" t="s">
         <v>108</v>
       </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
-      <c r="H2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="62"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="64"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="64"/>
+      <c r="D3" s="64"/>
+      <c r="E3" s="64"/>
+      <c r="F3" s="64"/>
+      <c r="G3" s="64"/>
+      <c r="H3" s="65"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="15"/>
@@ -1804,15 +1804,15 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="21"/>
-      <c r="C8" s="65" t="s">
+      <c r="C8" s="66" t="s">
         <v>96</v>
       </c>
-      <c r="D8" s="65"/>
+      <c r="D8" s="66"/>
       <c r="E8" s="22"/>
-      <c r="F8" s="65" t="s">
+      <c r="F8" s="66" t="s">
         <v>97</v>
       </c>
-      <c r="G8" s="65"/>
+      <c r="G8" s="66"/>
       <c r="H8" s="23"/>
     </row>
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -1994,11 +1994,11 @@
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="21"/>
-      <c r="C26" s="66"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="67"/>
-      <c r="F26" s="67"/>
-      <c r="G26" s="68"/>
+      <c r="C26" s="67"/>
+      <c r="D26" s="68"/>
+      <c r="E26" s="68"/>
+      <c r="F26" s="68"/>
+      <c r="G26" s="69"/>
       <c r="H26" s="23"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2098,61 +2098,61 @@
       <c r="X1" s="7"/>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="118" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="113" t="s">
+      <c r="B2" s="118" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="113" t="s">
+      <c r="C2" s="118" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="113" t="s">
+      <c r="D2" s="118" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="97" t="s">
-        <v>179</v>
+      <c r="E2" s="91" t="s">
+        <v>176</v>
       </c>
-      <c r="F2" s="88" t="s">
-        <v>188</v>
+      <c r="F2" s="98" t="s">
+        <v>185</v>
       </c>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="99" t="s">
-        <v>189</v>
+      <c r="G2" s="98"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="107" t="s">
+        <v>186</v>
       </c>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99" t="s">
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="107" t="s">
         <v>35</v>
       </c>
-      <c r="O2" s="99"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="103" t="s">
+      <c r="O2" s="107"/>
+      <c r="P2" s="107"/>
+      <c r="Q2" s="88" t="s">
         <v>38</v>
       </c>
-      <c r="R2" s="79" t="s">
+      <c r="R2" s="80" t="s">
         <v>61</v>
       </c>
-      <c r="S2" s="81"/>
-      <c r="T2" s="79" t="s">
-        <v>187</v>
+      <c r="S2" s="82"/>
+      <c r="T2" s="80" t="s">
+        <v>184</v>
       </c>
-      <c r="U2" s="80"/>
-      <c r="V2" s="81"/>
-      <c r="W2" s="96" t="s">
-        <v>186</v>
+      <c r="U2" s="81"/>
+      <c r="V2" s="82"/>
+      <c r="W2" s="106" t="s">
+        <v>183</v>
       </c>
-      <c r="X2" s="96"/>
+      <c r="X2" s="106"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="114"/>
-      <c r="B3" s="114"/>
-      <c r="C3" s="114"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="98"/>
+      <c r="A3" s="119"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="93"/>
       <c r="F3" s="45" t="s">
         <v>19</v>
       </c>
@@ -2160,7 +2160,7 @@
         <v>37</v>
       </c>
       <c r="H3" s="45" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="I3" s="41" t="s">
         <v>47</v>
@@ -2172,21 +2172,21 @@
         <v>37</v>
       </c>
       <c r="L3" s="40" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="M3" s="44" t="s">
         <v>47</v>
       </c>
       <c r="N3" s="40" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="O3" s="44" t="s">
         <v>36</v>
       </c>
       <c r="P3" s="56" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
-      <c r="Q3" s="104"/>
+      <c r="Q3" s="90"/>
       <c r="R3" s="47" t="s">
         <v>59</v>
       </c>
@@ -2200,13 +2200,13 @@
         <v>39</v>
       </c>
       <c r="V3" s="44" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="W3" s="40" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="X3" s="40" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.25">
@@ -7472,7 +7472,7 @@
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -7488,61 +7488,61 @@
       <c r="M1" s="14"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="118" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="113" t="s">
+      <c r="B2" s="118" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="113" t="s">
+      <c r="C2" s="118" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="113" t="s">
+      <c r="D2" s="118" t="s">
         <v>68</v>
       </c>
-      <c r="E2" s="103" t="s">
+      <c r="E2" s="88" t="s">
+        <v>188</v>
+      </c>
+      <c r="F2" s="88" t="s">
+        <v>189</v>
+      </c>
+      <c r="G2" s="88" t="s">
+        <v>190</v>
+      </c>
+      <c r="H2" s="120" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" s="89" t="s">
         <v>191</v>
       </c>
-      <c r="F2" s="103" t="s">
-        <v>192</v>
-      </c>
-      <c r="G2" s="103" t="s">
-        <v>193</v>
-      </c>
-      <c r="H2" s="116" t="s">
-        <v>44</v>
-      </c>
-      <c r="I2" s="115" t="s">
-        <v>194</v>
-      </c>
-      <c r="J2" s="116" t="s">
+      <c r="J2" s="120" t="s">
         <v>45</v>
       </c>
-      <c r="K2" s="116" t="s">
+      <c r="K2" s="120" t="s">
         <v>46</v>
       </c>
-      <c r="L2" s="91" t="s">
-        <v>186</v>
+      <c r="L2" s="101" t="s">
+        <v>183</v>
       </c>
-      <c r="M2" s="91"/>
+      <c r="M2" s="101"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="114"/>
-      <c r="B3" s="114"/>
-      <c r="C3" s="114"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="104"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="104"/>
-      <c r="J3" s="91"/>
-      <c r="K3" s="91"/>
+      <c r="A3" s="119"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="90"/>
+      <c r="G3" s="90"/>
+      <c r="H3" s="101"/>
+      <c r="I3" s="90"/>
+      <c r="J3" s="101"/>
+      <c r="K3" s="101"/>
       <c r="L3" s="40" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="M3" s="40" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -10548,11 +10548,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="BGDYvh08S3NYZIuspsRRCAicI1Gp8B4hCVX6TD3PYP3B6k2058cKh0vrrp9OQ+vPcDsnDczSdbeeSJcJFOUPXA==" saltValue="U5shOM/WfotH/IVdI6hz3g==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="12">
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="E2:E3"/>
@@ -10560,6 +10555,11 @@
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="H2:H3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F3 G2:G3 I2:I3 E2:E3 L3 M3" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -10640,10 +10640,10 @@
         <v>43</v>
       </c>
       <c r="J2" s="50" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K2" s="50" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -13278,7 +13278,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -13300,7 +13300,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F2" s="50" t="s">
         <v>91</v>
@@ -14980,117 +14980,117 @@
       <c r="X1" s="8"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="70" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="70" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69" t="s">
+      <c r="C2" s="70"/>
+      <c r="D2" s="70" t="s">
         <v>111</v>
       </c>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-      <c r="N2" s="69" t="s">
+      <c r="E2" s="70"/>
+      <c r="F2" s="70"/>
+      <c r="G2" s="70"/>
+      <c r="H2" s="70"/>
+      <c r="I2" s="70"/>
+      <c r="J2" s="70"/>
+      <c r="K2" s="70"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="70"/>
+      <c r="N2" s="70" t="s">
         <v>115</v>
       </c>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="69"/>
-      <c r="V2" s="69"/>
-      <c r="W2" s="69"/>
-      <c r="X2" s="69"/>
+      <c r="O2" s="70"/>
+      <c r="P2" s="70"/>
+      <c r="Q2" s="70"/>
+      <c r="R2" s="70"/>
+      <c r="S2" s="70"/>
+      <c r="T2" s="70"/>
+      <c r="U2" s="70"/>
+      <c r="V2" s="70"/>
+      <c r="W2" s="70"/>
+      <c r="X2" s="70"/>
       <c r="Y2" s="4"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="69"/>
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="72" t="s">
+      <c r="A3" s="70"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="73" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="78"/>
-      <c r="I3" s="72" t="s">
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="79"/>
+      <c r="I3" s="73" t="s">
         <v>53</v>
       </c>
-      <c r="J3" s="73"/>
-      <c r="K3" s="73"/>
-      <c r="L3" s="73"/>
-      <c r="M3" s="73"/>
-      <c r="N3" s="69"/>
-      <c r="O3" s="69"/>
-      <c r="P3" s="69"/>
-      <c r="Q3" s="69"/>
-      <c r="R3" s="69"/>
-      <c r="S3" s="69"/>
-      <c r="T3" s="69"/>
-      <c r="U3" s="69"/>
-      <c r="V3" s="69"/>
-      <c r="W3" s="69"/>
-      <c r="X3" s="69"/>
+      <c r="J3" s="74"/>
+      <c r="K3" s="74"/>
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="70"/>
+      <c r="O3" s="70"/>
+      <c r="P3" s="70"/>
+      <c r="Q3" s="70"/>
+      <c r="R3" s="70"/>
+      <c r="S3" s="70"/>
+      <c r="T3" s="70"/>
+      <c r="U3" s="70"/>
+      <c r="V3" s="70"/>
+      <c r="W3" s="70"/>
+      <c r="X3" s="70"/>
       <c r="Y3" s="4"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="69"/>
-      <c r="B4" s="69"/>
-      <c r="C4" s="69"/>
-      <c r="D4" s="70" t="s">
+      <c r="A4" s="70"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="71" t="s">
         <v>112</v>
       </c>
-      <c r="E4" s="71"/>
-      <c r="F4" s="70" t="s">
+      <c r="E4" s="72"/>
+      <c r="F4" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="G4" s="71"/>
-      <c r="H4" s="76" t="s">
+      <c r="G4" s="72"/>
+      <c r="H4" s="77" t="s">
         <v>55</v>
       </c>
-      <c r="I4" s="74" t="s">
+      <c r="I4" s="75" t="s">
         <v>112</v>
       </c>
-      <c r="J4" s="75"/>
-      <c r="K4" s="70" t="s">
+      <c r="J4" s="76"/>
+      <c r="K4" s="71" t="s">
         <v>113</v>
       </c>
-      <c r="L4" s="71"/>
-      <c r="M4" s="76" t="s">
+      <c r="L4" s="72"/>
+      <c r="M4" s="77" t="s">
         <v>55</v>
       </c>
-      <c r="N4" s="69" t="s">
+      <c r="N4" s="70" t="s">
         <v>116</v>
       </c>
-      <c r="O4" s="69"/>
-      <c r="P4" s="69" t="s">
+      <c r="O4" s="70"/>
+      <c r="P4" s="70" t="s">
         <v>117</v>
       </c>
-      <c r="Q4" s="69"/>
-      <c r="R4" s="69"/>
-      <c r="S4" s="69"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="79" t="s">
+      <c r="Q4" s="70"/>
+      <c r="R4" s="70"/>
+      <c r="S4" s="70"/>
+      <c r="T4" s="70"/>
+      <c r="U4" s="80" t="s">
         <v>118</v>
       </c>
-      <c r="V4" s="80"/>
-      <c r="W4" s="80"/>
-      <c r="X4" s="81"/>
+      <c r="V4" s="81"/>
+      <c r="W4" s="81"/>
+      <c r="X4" s="82"/>
     </row>
     <row r="5" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="69"/>
+      <c r="A5" s="70"/>
       <c r="B5" s="41" t="s">
         <v>92</v>
       </c>
@@ -15109,7 +15109,7 @@
       <c r="G5" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="H5" s="77"/>
+      <c r="H5" s="78"/>
       <c r="I5" s="40" t="s">
         <v>114</v>
       </c>
@@ -15122,7 +15122,7 @@
       <c r="L5" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="M5" s="77"/>
+      <c r="M5" s="78"/>
       <c r="N5" s="41" t="s">
         <v>5</v>
       </c>
@@ -20334,7 +20334,7 @@
       <c r="X204" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="RdNrOAn/lQMbMlrvotSd6e7DAP6LRqnMQsSQdK2ijNoYLV6uZuPnsrPuGGdEV+gbuZ9hwJUmPp3VbLE6xYZ72A==" saltValue="8ZiNB57QGOGYw7UGazEnig==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="kuraIphfBcjZ2nHiigUoBx9E5Jz+h7+0bz47tq+vlXnhlBdiMjPoHdZkgU9MsIUPHl1S+9z35QqCZfKvYAu2VA==" saltValue="iN+qBwmj3LDfsG6tTAfGtg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="15">
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="N4:O4"/>
@@ -20419,87 +20419,87 @@
       <c r="P1" s="8"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="85" t="s">
+      <c r="B2" s="95" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="86"/>
-      <c r="D2" s="86"/>
-      <c r="E2" s="86"/>
-      <c r="F2" s="87"/>
+      <c r="C2" s="96"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="97"/>
       <c r="G2" s="83" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="117"/>
-      <c r="I2" s="84"/>
-      <c r="J2" s="103" t="s">
-        <v>201</v>
+      <c r="H2" s="84"/>
+      <c r="I2" s="85"/>
+      <c r="J2" s="88" t="s">
+        <v>198</v>
       </c>
-      <c r="K2" s="97" t="s">
+      <c r="K2" s="91" t="s">
         <v>123</v>
       </c>
-      <c r="L2" s="85" t="s">
+      <c r="L2" s="95" t="s">
         <v>107</v>
       </c>
-      <c r="M2" s="86"/>
-      <c r="N2" s="86"/>
-      <c r="O2" s="86"/>
-      <c r="P2" s="87"/>
+      <c r="M2" s="96"/>
+      <c r="N2" s="96"/>
+      <c r="O2" s="96"/>
+      <c r="P2" s="97"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="82"/>
-      <c r="B3" s="69" t="s">
+      <c r="A3" s="94"/>
+      <c r="B3" s="70" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="95" t="s">
-        <v>199</v>
+      <c r="C3" s="105" t="s">
+        <v>196</v>
       </c>
-      <c r="D3" s="69" t="s">
+      <c r="D3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="90" t="s">
+      <c r="E3" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="96" t="s">
+      <c r="F3" s="106" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="92" t="s">
+      <c r="G3" s="102" t="s">
         <v>114</v>
       </c>
-      <c r="H3" s="93" t="s">
+      <c r="H3" s="103" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="118" t="s">
-        <v>200</v>
+      <c r="I3" s="86" t="s">
+        <v>197</v>
       </c>
-      <c r="J3" s="115"/>
-      <c r="K3" s="109"/>
-      <c r="L3" s="88" t="s">
+      <c r="J3" s="89"/>
+      <c r="K3" s="92"/>
+      <c r="L3" s="98" t="s">
         <v>124</v>
       </c>
-      <c r="M3" s="88"/>
-      <c r="N3" s="88" t="s">
+      <c r="M3" s="98"/>
+      <c r="N3" s="98" t="s">
         <v>125</v>
       </c>
-      <c r="O3" s="88"/>
-      <c r="P3" s="89" t="s">
+      <c r="O3" s="98"/>
+      <c r="P3" s="99" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="77"/>
-      <c r="B4" s="69"/>
-      <c r="C4" s="95"/>
-      <c r="D4" s="69"/>
-      <c r="E4" s="91"/>
-      <c r="F4" s="96"/>
-      <c r="G4" s="92"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="119"/>
-      <c r="J4" s="104"/>
-      <c r="K4" s="98"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="105"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="101"/>
+      <c r="F4" s="106"/>
+      <c r="G4" s="102"/>
+      <c r="H4" s="104"/>
+      <c r="I4" s="87"/>
+      <c r="J4" s="90"/>
+      <c r="K4" s="93"/>
       <c r="L4" s="41" t="s">
         <v>3</v>
       </c>
@@ -20512,7 +20512,7 @@
       <c r="O4" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="P4" s="89"/>
+      <c r="P4" s="99"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -24115,13 +24115,8 @@
       <c r="P204" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="bfwcZBaZ/SEpauMzvnRVd4A28z1cS1DkAIJnucm/zY9+/BV9GBCfb1hNoT3BC7EfOAKKln0AkgUeOJAdZmGg0A==" saltValue="vcjCV3XhbNlYrDAn3hdkSQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="O3vPd5vM4N/Qh7B6qHZd426iarnVuOzAMFoRd4rVrG3TYR7D813UKsBbjt/FHVt++j2pUvdy4VeHDazqXO/KsQ==" saltValue="x4iNhhhTzYRRYu28b3Rbjw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J2:J4"/>
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="A2:A4"/>
     <mergeCell ref="L2:P2"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="P3:P4"/>
@@ -24134,6 +24129,11 @@
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J2:J4"/>
+    <mergeCell ref="K2:K4"/>
+    <mergeCell ref="A2:A4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M4 O4 H3:H4 J2:K2" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -24193,47 +24193,47 @@
       <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="98" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88" t="s">
+      <c r="C2" s="98"/>
+      <c r="D2" s="98"/>
+      <c r="E2" s="98"/>
+      <c r="F2" s="98"/>
+      <c r="G2" s="98" t="s">
         <v>128</v>
       </c>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
+      <c r="H2" s="98"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="98"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="82"/>
-      <c r="B3" s="72" t="s">
+      <c r="A3" s="94"/>
+      <c r="B3" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="76" t="s">
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="77" t="s">
         <v>55</v>
       </c>
-      <c r="G3" s="72" t="s">
+      <c r="G3" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="78"/>
-      <c r="K3" s="76" t="s">
+      <c r="H3" s="74"/>
+      <c r="I3" s="74"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="77" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="77"/>
+      <c r="A4" s="78"/>
       <c r="B4" s="40" t="s">
         <v>114</v>
       </c>
@@ -24246,7 +24246,7 @@
       <c r="E4" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="F4" s="77"/>
+      <c r="F4" s="78"/>
       <c r="G4" s="40" t="s">
         <v>114</v>
       </c>
@@ -24259,7 +24259,7 @@
       <c r="J4" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="K4" s="77"/>
+      <c r="K4" s="78"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -26981,175 +26981,175 @@
       <c r="AO1" s="7"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="80" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="80"/>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="80"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="80"/>
-      <c r="O2" s="80"/>
-      <c r="P2" s="80"/>
-      <c r="Q2" s="80"/>
-      <c r="R2" s="80"/>
-      <c r="S2" s="80"/>
-      <c r="T2" s="81"/>
-      <c r="U2" s="79" t="s">
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="81"/>
+      <c r="N2" s="81"/>
+      <c r="O2" s="81"/>
+      <c r="P2" s="81"/>
+      <c r="Q2" s="81"/>
+      <c r="R2" s="81"/>
+      <c r="S2" s="81"/>
+      <c r="T2" s="82"/>
+      <c r="U2" s="80" t="s">
         <v>155</v>
       </c>
-      <c r="V2" s="80"/>
-      <c r="W2" s="80"/>
-      <c r="X2" s="80"/>
-      <c r="Y2" s="80"/>
-      <c r="Z2" s="80"/>
-      <c r="AA2" s="80"/>
-      <c r="AB2" s="80"/>
-      <c r="AC2" s="80"/>
-      <c r="AD2" s="80"/>
-      <c r="AE2" s="80"/>
-      <c r="AF2" s="80"/>
-      <c r="AG2" s="81"/>
-      <c r="AH2" s="79" t="s">
+      <c r="V2" s="81"/>
+      <c r="W2" s="81"/>
+      <c r="X2" s="81"/>
+      <c r="Y2" s="81"/>
+      <c r="Z2" s="81"/>
+      <c r="AA2" s="81"/>
+      <c r="AB2" s="81"/>
+      <c r="AC2" s="81"/>
+      <c r="AD2" s="81"/>
+      <c r="AE2" s="81"/>
+      <c r="AF2" s="81"/>
+      <c r="AG2" s="82"/>
+      <c r="AH2" s="80" t="s">
         <v>142</v>
       </c>
-      <c r="AI2" s="80"/>
-      <c r="AJ2" s="80"/>
-      <c r="AK2" s="80"/>
-      <c r="AL2" s="80"/>
-      <c r="AM2" s="80"/>
-      <c r="AN2" s="80"/>
-      <c r="AO2" s="81"/>
+      <c r="AI2" s="81"/>
+      <c r="AJ2" s="81"/>
+      <c r="AK2" s="81"/>
+      <c r="AL2" s="81"/>
+      <c r="AM2" s="81"/>
+      <c r="AN2" s="81"/>
+      <c r="AO2" s="82"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="82"/>
-      <c r="B3" s="90" t="s">
-        <v>202</v>
+      <c r="A3" s="94"/>
+      <c r="B3" s="100" t="s">
+        <v>199</v>
       </c>
-      <c r="C3" s="100" t="s">
+      <c r="C3" s="108" t="s">
+        <v>200</v>
+      </c>
+      <c r="D3" s="88" t="s">
+        <v>129</v>
+      </c>
+      <c r="E3" s="107" t="s">
+        <v>130</v>
+      </c>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107" t="s">
+        <v>131</v>
+      </c>
+      <c r="I3" s="107"/>
+      <c r="J3" s="107"/>
+      <c r="K3" s="109" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="103" t="s">
-        <v>129</v>
-      </c>
-      <c r="E3" s="99" t="s">
-        <v>130</v>
-      </c>
-      <c r="F3" s="99"/>
-      <c r="G3" s="99"/>
-      <c r="H3" s="99" t="s">
-        <v>131</v>
-      </c>
-      <c r="I3" s="99"/>
-      <c r="J3" s="99"/>
-      <c r="K3" s="101" t="s">
-        <v>206</v>
-      </c>
-      <c r="L3" s="96" t="s">
+      <c r="L3" s="106" t="s">
         <v>136</v>
       </c>
-      <c r="M3" s="96"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="96"/>
-      <c r="P3" s="99" t="s">
+      <c r="M3" s="106"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="106"/>
+      <c r="P3" s="107" t="s">
         <v>137</v>
       </c>
-      <c r="Q3" s="99"/>
-      <c r="R3" s="99"/>
-      <c r="S3" s="96" t="s">
+      <c r="Q3" s="107"/>
+      <c r="R3" s="107"/>
+      <c r="S3" s="106" t="s">
         <v>22</v>
       </c>
-      <c r="T3" s="96"/>
-      <c r="U3" s="99" t="s">
+      <c r="T3" s="106"/>
+      <c r="U3" s="107" t="s">
         <v>141</v>
       </c>
-      <c r="V3" s="99" t="s">
+      <c r="V3" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="W3" s="99" t="s">
+      <c r="W3" s="107" t="s">
         <v>34</v>
       </c>
-      <c r="X3" s="99" t="s">
+      <c r="X3" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="Y3" s="99" t="s">
+      <c r="Y3" s="107" t="s">
         <v>25</v>
       </c>
-      <c r="Z3" s="99" t="s">
+      <c r="Z3" s="107" t="s">
         <v>26</v>
       </c>
-      <c r="AA3" s="99" t="s">
+      <c r="AA3" s="107" t="s">
         <v>27</v>
       </c>
-      <c r="AB3" s="99" t="s">
+      <c r="AB3" s="107" t="s">
         <v>28</v>
       </c>
-      <c r="AC3" s="99" t="s">
+      <c r="AC3" s="107" t="s">
         <v>29</v>
       </c>
-      <c r="AD3" s="99" t="s">
+      <c r="AD3" s="107" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="99" t="s">
+      <c r="AE3" s="107" t="s">
         <v>31</v>
       </c>
-      <c r="AF3" s="99" t="s">
+      <c r="AF3" s="107" t="s">
         <v>32</v>
       </c>
-      <c r="AG3" s="99" t="s">
+      <c r="AG3" s="107" t="s">
         <v>33</v>
       </c>
-      <c r="AH3" s="96" t="s">
+      <c r="AH3" s="106" t="s">
         <v>151</v>
       </c>
-      <c r="AI3" s="96"/>
-      <c r="AJ3" s="96" t="s">
+      <c r="AI3" s="106"/>
+      <c r="AJ3" s="106" t="s">
         <v>152</v>
       </c>
-      <c r="AK3" s="96"/>
-      <c r="AL3" s="96" t="s">
+      <c r="AK3" s="106"/>
+      <c r="AL3" s="106" t="s">
         <v>153</v>
       </c>
-      <c r="AM3" s="96"/>
-      <c r="AN3" s="96" t="s">
+      <c r="AM3" s="106"/>
+      <c r="AN3" s="106" t="s">
         <v>154</v>
       </c>
-      <c r="AO3" s="96"/>
+      <c r="AO3" s="106"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A4" s="77"/>
-      <c r="B4" s="91"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="104"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="101"/>
+      <c r="C4" s="75"/>
+      <c r="D4" s="90"/>
       <c r="E4" s="50" t="s">
         <v>20</v>
       </c>
       <c r="F4" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="G4" s="120" t="s">
-        <v>204</v>
+      <c r="G4" s="59" t="s">
+        <v>201</v>
       </c>
-      <c r="H4" s="120" t="s">
+      <c r="H4" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="120" t="s">
+      <c r="I4" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="120" t="s">
-        <v>204</v>
+      <c r="J4" s="59" t="s">
+        <v>201</v>
       </c>
-      <c r="K4" s="102"/>
+      <c r="K4" s="110"/>
       <c r="L4" s="40" t="s">
         <v>132</v>
       </c>
@@ -27175,21 +27175,21 @@
         <v>18</v>
       </c>
       <c r="T4" s="51" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
-      <c r="U4" s="99"/>
-      <c r="V4" s="99"/>
-      <c r="W4" s="99"/>
-      <c r="X4" s="99"/>
-      <c r="Y4" s="99"/>
-      <c r="Z4" s="99"/>
-      <c r="AA4" s="99"/>
-      <c r="AB4" s="99"/>
-      <c r="AC4" s="99"/>
-      <c r="AD4" s="99"/>
-      <c r="AE4" s="99"/>
-      <c r="AF4" s="99"/>
-      <c r="AG4" s="99"/>
+      <c r="U4" s="107"/>
+      <c r="V4" s="107"/>
+      <c r="W4" s="107"/>
+      <c r="X4" s="107"/>
+      <c r="Y4" s="107"/>
+      <c r="Z4" s="107"/>
+      <c r="AA4" s="107"/>
+      <c r="AB4" s="107"/>
+      <c r="AC4" s="107"/>
+      <c r="AD4" s="107"/>
+      <c r="AE4" s="107"/>
+      <c r="AF4" s="107"/>
+      <c r="AG4" s="107"/>
       <c r="AH4" s="52" t="s">
         <v>143</v>
       </c>
@@ -35816,22 +35816,8 @@
       <c r="AO204" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="JacJblqysVn4VlodL3cUZIOB9Nry7+tfevwii5NIAWEA2sxBjghxk+OgRjF/SuUA1DLt+bB7HT5LyH8oN4ka6Q==" saltValue="mhMw97y/oUl8/Qxr6rgwXQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="QEQd2x0BKHbPsCCaNKPWr4HTNrPyaNjaEkhTFqmOR7qEW7lhdXdsDzn/18LwB+BtaIdU1miotO/Ku4vF690czA==" saltValue="EPC4iVtkM6J5UbKwOSWluA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
-    <mergeCell ref="AC3:AC4"/>
-    <mergeCell ref="AG3:AG4"/>
-    <mergeCell ref="L3:O3"/>
-    <mergeCell ref="AL3:AM3"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AJ3:AK3"/>
-    <mergeCell ref="AF3:AF4"/>
-    <mergeCell ref="AE3:AE4"/>
-    <mergeCell ref="AD3:AD4"/>
-    <mergeCell ref="W3:W4"/>
-    <mergeCell ref="AA3:AA4"/>
-    <mergeCell ref="Z3:Z4"/>
-    <mergeCell ref="Y3:Y4"/>
-    <mergeCell ref="X3:X4"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="B2:T2"/>
     <mergeCell ref="U2:AG2"/>
@@ -35848,6 +35834,20 @@
     <mergeCell ref="V3:V4"/>
     <mergeCell ref="AN3:AO3"/>
     <mergeCell ref="D3:D4"/>
+    <mergeCell ref="AC3:AC4"/>
+    <mergeCell ref="AG3:AG4"/>
+    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="AH3:AI3"/>
+    <mergeCell ref="AJ3:AK3"/>
+    <mergeCell ref="AF3:AF4"/>
+    <mergeCell ref="AE3:AE4"/>
+    <mergeCell ref="AD3:AD4"/>
+    <mergeCell ref="W3:W4"/>
+    <mergeCell ref="AA3:AA4"/>
+    <mergeCell ref="Z3:Z4"/>
+    <mergeCell ref="Y3:Y4"/>
+    <mergeCell ref="X3:X4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN4 D3:D4 L4 M4 N4 O4 P4 Q4 R4 AH4 AI4 AJ4 AK4 AL4 AM4 AO4" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -35888,7 +35888,7 @@
     <col min="2" max="3" width="18.5703125" style="3" customWidth="1"/>
     <col min="9" max="9" width="12.5703125" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" customWidth="1"/>
-    <col min="12" max="12" width="20.5703125" customWidth="1"/>
+    <col min="12" max="12" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
@@ -35908,98 +35908,98 @@
       <c r="L1" s="9"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="80" t="s">
         <v>157</v>
       </c>
-      <c r="C2" s="81"/>
-      <c r="D2" s="79" t="s">
+      <c r="C2" s="82"/>
+      <c r="D2" s="80" t="s">
         <v>158</v>
       </c>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
-      <c r="J2" s="80"/>
-      <c r="K2" s="80"/>
-      <c r="L2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="82"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="82"/>
-      <c r="B3" s="96" t="s">
+      <c r="A3" s="94"/>
+      <c r="B3" s="106" t="s">
         <v>70</v>
       </c>
-      <c r="C3" s="96" t="s">
+      <c r="C3" s="106" t="s">
         <v>71</v>
       </c>
-      <c r="D3" s="96" t="s">
+      <c r="D3" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="96"/>
-      <c r="F3" s="96"/>
-      <c r="G3" s="96"/>
-      <c r="H3" s="96" t="s">
+      <c r="E3" s="106"/>
+      <c r="F3" s="106"/>
+      <c r="G3" s="106"/>
+      <c r="H3" s="106" t="s">
         <v>159</v>
       </c>
-      <c r="I3" s="96"/>
-      <c r="J3" s="96"/>
-      <c r="K3" s="96"/>
-      <c r="L3" s="96" t="s">
+      <c r="I3" s="106"/>
+      <c r="J3" s="106"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="106" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="94"/>
+      <c r="B4" s="106"/>
+      <c r="C4" s="106"/>
+      <c r="D4" s="106" t="s">
+        <v>207</v>
+      </c>
+      <c r="E4" s="106"/>
+      <c r="F4" s="106" t="s">
+        <v>208</v>
+      </c>
+      <c r="G4" s="106"/>
+      <c r="H4" s="106" t="s">
+        <v>161</v>
+      </c>
+      <c r="I4" s="106"/>
+      <c r="J4" s="106" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="82"/>
-      <c r="B4" s="96"/>
-      <c r="C4" s="96"/>
-      <c r="D4" s="96" t="s">
-        <v>164</v>
-      </c>
-      <c r="E4" s="96"/>
-      <c r="F4" s="96" t="s">
-        <v>163</v>
-      </c>
-      <c r="G4" s="96"/>
-      <c r="H4" s="96" t="s">
-        <v>162</v>
-      </c>
-      <c r="I4" s="96"/>
-      <c r="J4" s="96" t="s">
-        <v>161</v>
-      </c>
-      <c r="K4" s="96"/>
-      <c r="L4" s="96"/>
+      <c r="K4" s="106"/>
+      <c r="L4" s="106"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="77"/>
-      <c r="B5" s="96"/>
-      <c r="C5" s="96"/>
-      <c r="D5" s="44" t="s">
+      <c r="A5" s="78"/>
+      <c r="B5" s="106"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="51" t="s">
-        <v>205</v>
+      <c r="E5" s="57" t="s">
+        <v>202</v>
       </c>
-      <c r="F5" s="44" t="s">
+      <c r="F5" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="51" t="s">
-        <v>205</v>
+      <c r="G5" s="57" t="s">
+        <v>202</v>
       </c>
-      <c r="H5" s="44" t="s">
+      <c r="H5" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="51" t="s">
-        <v>205</v>
+      <c r="I5" s="57" t="s">
+        <v>202</v>
       </c>
-      <c r="J5" s="44" t="s">
+      <c r="J5" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="K5" s="51" t="s">
-        <v>205</v>
+      <c r="K5" s="57" t="s">
+        <v>202</v>
       </c>
       <c r="L5" s="44" t="s">
         <v>73</v>
@@ -38806,7 +38806,7 @@
       <c r="L205" s="12"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="OIA2juXsQVr9S2oP2mybawOifHzCkVXtWAdDfZJ2K3RMDe4SYTT0Jit/7m2eczthvGnOsPbITjE52MRfvCrPMA==" saltValue="DWrHcNm1oKnbWvyYitlxgA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="t43DLs+s5NR3jDRJjGFNrGXdd0zh6ig4+D6iaOgaTgwQCtZa1klKK01BY/Aj5GsBKodHv1cSKsVMcorIrbKhgw==" saltValue="DsbiSSsnv29CJQyWru+yRQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="12">
     <mergeCell ref="D2:L2"/>
     <mergeCell ref="A2:A5"/>
@@ -38878,91 +38878,91 @@
       <c r="V1" s="7"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="72" t="s">
-        <v>165</v>
+      <c r="C2" s="73" t="s">
+        <v>162</v>
       </c>
-      <c r="D2" s="73"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="100" t="s">
-        <v>166</v>
+      <c r="D2" s="74"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="108" t="s">
+        <v>163</v>
       </c>
-      <c r="G2" s="106"/>
-      <c r="H2" s="106"/>
-      <c r="I2" s="106"/>
-      <c r="J2" s="97" t="s">
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="91" t="s">
         <v>89</v>
       </c>
-      <c r="K2" s="108" t="s">
+      <c r="K2" s="113" t="s">
+        <v>168</v>
+      </c>
+      <c r="L2" s="106" t="s">
+        <v>75</v>
+      </c>
+      <c r="M2" s="99" t="s">
+        <v>76</v>
+      </c>
+      <c r="N2" s="106" t="s">
+        <v>77</v>
+      </c>
+      <c r="O2" s="80"/>
+      <c r="P2" s="77" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q2" s="82" t="s">
+        <v>79</v>
+      </c>
+      <c r="R2" s="106" t="s">
+        <v>169</v>
+      </c>
+      <c r="S2" s="106"/>
+      <c r="T2" s="106"/>
+      <c r="U2" s="106"/>
+      <c r="V2" s="106"/>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A3" s="94"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="114" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="73" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="79"/>
+      <c r="F3" s="75"/>
+      <c r="G3" s="112"/>
+      <c r="H3" s="112"/>
+      <c r="I3" s="112"/>
+      <c r="J3" s="92"/>
+      <c r="K3" s="113"/>
+      <c r="L3" s="106"/>
+      <c r="M3" s="99"/>
+      <c r="N3" s="106"/>
+      <c r="O3" s="80"/>
+      <c r="P3" s="94"/>
+      <c r="Q3" s="82"/>
+      <c r="R3" s="107" t="s">
+        <v>80</v>
+      </c>
+      <c r="S3" s="106" t="s">
+        <v>170</v>
+      </c>
+      <c r="T3" s="106"/>
+      <c r="U3" s="106" t="s">
         <v>171</v>
       </c>
-      <c r="L2" s="96" t="s">
-        <v>75</v>
-      </c>
-      <c r="M2" s="89" t="s">
-        <v>76</v>
-      </c>
-      <c r="N2" s="96" t="s">
-        <v>77</v>
-      </c>
-      <c r="O2" s="79"/>
-      <c r="P2" s="76" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q2" s="81" t="s">
-        <v>79</v>
-      </c>
-      <c r="R2" s="96" t="s">
-        <v>172</v>
-      </c>
-      <c r="S2" s="96"/>
-      <c r="T2" s="96"/>
-      <c r="U2" s="96"/>
-      <c r="V2" s="96"/>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="82"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="105" t="s">
-        <v>55</v>
-      </c>
-      <c r="D3" s="72" t="s">
-        <v>54</v>
-      </c>
-      <c r="E3" s="78"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="107"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="109"/>
-      <c r="K3" s="108"/>
-      <c r="L3" s="96"/>
-      <c r="M3" s="89"/>
-      <c r="N3" s="96"/>
-      <c r="O3" s="79"/>
-      <c r="P3" s="82"/>
-      <c r="Q3" s="81"/>
-      <c r="R3" s="99" t="s">
-        <v>80</v>
-      </c>
-      <c r="S3" s="96" t="s">
-        <v>173</v>
-      </c>
-      <c r="T3" s="96"/>
-      <c r="U3" s="96" t="s">
-        <v>174</v>
-      </c>
-      <c r="V3" s="96"/>
+      <c r="V3" s="106"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A4" s="77"/>
-      <c r="B4" s="77"/>
-      <c r="C4" s="70"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="71"/>
       <c r="D4" s="41" t="s">
         <v>0</v>
       </c>
@@ -38970,30 +38970,30 @@
         <v>1</v>
       </c>
       <c r="F4" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="G4" s="40" t="s">
+        <v>165</v>
+      </c>
+      <c r="H4" s="40" t="s">
+        <v>166</v>
+      </c>
+      <c r="I4" s="54" t="s">
         <v>167</v>
       </c>
-      <c r="G4" s="40" t="s">
-        <v>168</v>
-      </c>
-      <c r="H4" s="40" t="s">
-        <v>169</v>
-      </c>
-      <c r="I4" s="54" t="s">
-        <v>170</v>
-      </c>
-      <c r="J4" s="98"/>
-      <c r="K4" s="108"/>
-      <c r="L4" s="96"/>
-      <c r="M4" s="89"/>
+      <c r="J4" s="93"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="106"/>
+      <c r="M4" s="99"/>
       <c r="N4" s="46" t="s">
         <v>81</v>
       </c>
       <c r="O4" s="53" t="s">
         <v>82</v>
       </c>
-      <c r="P4" s="77"/>
-      <c r="Q4" s="81"/>
-      <c r="R4" s="99"/>
+      <c r="P4" s="78"/>
+      <c r="Q4" s="82"/>
+      <c r="R4" s="107"/>
       <c r="S4" s="50" t="s">
         <v>83</v>
       </c>
@@ -39001,10 +39001,10 @@
         <v>84</v>
       </c>
       <c r="U4" s="43" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="V4" s="43" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
@@ -43808,9 +43808,14 @@
       <c r="V204" s="12"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="HegNjEUG0JGCK7Em0JYKFfbaDXofSI/eoHWk8rSNZhCuxxgrRfFxzqmKDw+rgM8g2AEjX7hW0V65tqpclq3eIA==" saltValue="dNae070C6OTNQ7yDYKjQHg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="DH4pbwpBCgOVxJ9KK8YMUqoGVi4hN4h0sZoI4bzxOwYd6s3rgpQnpSBPYhaWIv/lB5Wz8frrYtZ8i1ITmBBXew==" saltValue="K66eZwZ2YOSlOz/j5lhrvw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="17">
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
     <mergeCell ref="R2:V2"/>
     <mergeCell ref="R3:R4"/>
     <mergeCell ref="S3:T3"/>
@@ -43823,11 +43828,6 @@
     <mergeCell ref="N2:O3"/>
     <mergeCell ref="J2:J4"/>
     <mergeCell ref="P2:P4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="A2:A4"/>
-    <mergeCell ref="B2:B4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K4 I4 F4 G4 H4 U4 V4" xr:uid="{7CB5582D-4A36-46D9-AA38-ED8FA154223A}">
@@ -43865,14 +43865,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="110" t="s">
-        <v>207</v>
+      <c r="A1" s="115" t="s">
+        <v>204</v>
       </c>
-      <c r="B1" s="110"/>
-      <c r="C1" s="110"/>
-      <c r="D1" s="110"/>
-      <c r="E1" s="110"/>
-      <c r="F1" s="110"/>
+      <c r="B1" s="115"/>
+      <c r="C1" s="115"/>
+      <c r="D1" s="115"/>
+      <c r="E1" s="115"/>
+      <c r="F1" s="115"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="41" t="s">
@@ -43885,10 +43885,10 @@
         <v>85</v>
       </c>
       <c r="D2" s="45" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E2" s="41" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="F2" s="41" t="s">
         <v>86</v>
@@ -45495,7 +45495,7 @@
       <c r="F202" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="kviV1SZRnQko8ezco/44rWDpyPVJvrbA6GYXl6ikqHqao1OSEmfHNyEdJQTk0awshCQvmkR1NuK7VUgYncNMcQ==" saltValue="h3WPTOpyhj/BFNU0j0oJPA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="FN5XjCkfoJMzNB3xxSMxF5fTBE47EIi4lyn8towZTKfC6UgUKWnx0SjqUB0dvx+fMO28pkDJTfvcixTOGR4P/g==" saltValue="PlngWBfIMMySzBcBNAG5ng==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -45549,59 +45549,59 @@
       <c r="L1" s="8"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="76" t="s">
+      <c r="A2" s="77" t="s">
         <v>65</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="77" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="76" t="s">
+      <c r="C2" s="77" t="s">
         <v>67</v>
       </c>
-      <c r="D2" s="97" t="s">
-        <v>177</v>
+      <c r="D2" s="91" t="s">
+        <v>174</v>
       </c>
-      <c r="E2" s="111" t="s">
+      <c r="E2" s="116" t="s">
         <v>63</v>
       </c>
-      <c r="F2" s="112"/>
-      <c r="G2" s="97" t="s">
-        <v>179</v>
+      <c r="F2" s="117"/>
+      <c r="G2" s="91" t="s">
+        <v>176</v>
       </c>
-      <c r="H2" s="76" t="s">
-        <v>178</v>
+      <c r="H2" s="77" t="s">
+        <v>175</v>
       </c>
-      <c r="I2" s="72" t="s">
+      <c r="I2" s="73" t="s">
         <v>35</v>
       </c>
-      <c r="J2" s="73"/>
-      <c r="K2" s="73"/>
-      <c r="L2" s="78"/>
+      <c r="J2" s="74"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="79"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="77"/>
-      <c r="B3" s="77"/>
-      <c r="C3" s="77"/>
-      <c r="D3" s="98"/>
+      <c r="A3" s="78"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="93"/>
       <c r="E3" s="49" t="s">
         <v>19</v>
       </c>
       <c r="F3" s="49" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="98"/>
-      <c r="H3" s="77"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="78"/>
       <c r="I3" s="49" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="J3" s="48" t="s">
         <v>18</v>
       </c>
       <c r="K3" s="55" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="L3" s="49" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -48405,7 +48405,7 @@
       <c r="L203" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="UKy/9FtM0qE00vQznJsrAB6qNs4GW8BQPbqIcWB/O1BV/Zo2g6FqcmjtYLjBLHAOlTWuzmOBMkW75s7THcQJ1g==" saltValue="oLVNnQ9vZNGxIvvoNMp/5A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="BGhIRZNXhHaWJYiU7Xlb4CwauylZ3rZdEH/3xrzCZbWI3WIAAuTgy6kEv7npV936xqH+cyCevlkWl26lZ9H7aw==" saltValue="ykBltnH/IwlrQJ7k84BDuA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="8">
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="D2:D3"/>

</xml_diff>

<commit_message>
inclusion of logic response code lists in LL, PS, and 3DA form descriptions
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -11,7 +11,7 @@
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCD133D-7224-4E04-93EA-25A03D08B21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="c5/ou8Cml7ZkaDU47Tuu3WsAbYP19DC42wRzPBn3vsHWJE2MFn5j3m9vhk0UNMu/icNe5bym2Fttv6xJI1ZSAw==" workbookSaltValue="pG4NehU6lkQVWVHx3qNlvg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="5" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -1205,6 +1205,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
@@ -1281,14 +1289,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1301,6 +1301,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1310,9 +1313,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2012,15 +2012,15 @@
       <c r="D1" s="109" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="78" t="s">
+      <c r="E1" s="80" t="s">
         <v>163</v>
       </c>
-      <c r="F1" s="85" t="s">
+      <c r="F1" s="87" t="s">
         <v>169</v>
       </c>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
+      <c r="G1" s="87"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
       <c r="J1" s="99" t="s">
         <v>170</v>
       </c>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="O1" s="99"/>
       <c r="P1" s="99"/>
-      <c r="Q1" s="75" t="s">
+      <c r="Q1" s="77" t="s">
         <v>38</v>
       </c>
       <c r="R1" s="72" t="s">
@@ -2050,7 +2050,7 @@
       <c r="B2" s="110"/>
       <c r="C2" s="110"/>
       <c r="D2" s="110"/>
-      <c r="E2" s="80"/>
+      <c r="E2" s="82"/>
       <c r="F2" s="36" t="s">
         <v>19</v>
       </c>
@@ -2084,7 +2084,7 @@
       <c r="P2" s="45" t="s">
         <v>167</v>
       </c>
-      <c r="Q2" s="77"/>
+      <c r="Q2" s="79"/>
       <c r="R2" s="38" t="s">
         <v>53</v>
       </c>
@@ -6904,17 +6904,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="F0tc7B77v7QjLsOz0RLL7MWtNCPBw2o4Z9f2YID1JxL/5n/IHv5nh1k9azF4NV4h1VsWAZfQTfWlFcYB76PlMA==" saltValue="n01OBaL5NKfbkpK2LmYd9A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="Q1:Q2"/>
     <mergeCell ref="T1:V1"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="N1:P1"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="Q1:Q2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E2 F2 H2 J2 L2 N2 Q1:Q2" xr:uid="{CF79E0B9-452F-42D7-82F9-4325C7CCE12E}">
@@ -6974,19 +6974,19 @@
       <c r="D1" s="109" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="75" t="s">
+      <c r="E1" s="77" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="75" t="s">
+      <c r="F1" s="77" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="75" t="s">
+      <c r="G1" s="77" t="s">
         <v>173</v>
       </c>
       <c r="H1" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="76" t="s">
+      <c r="I1" s="78" t="s">
         <v>174</v>
       </c>
       <c r="J1" s="111" t="s">
@@ -7001,13 +7001,13 @@
       <c r="B2" s="110"/>
       <c r="C2" s="110"/>
       <c r="D2" s="110"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="77"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="90"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="90"/>
+      <c r="K2" s="90"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -9612,17 +9612,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="7AjhL+fqXAsFucLZgoF2uPzgppBK+T/XTUzkX/JwpgqEiyXl3lYNCR44gk+4O6ySKgm58zlH7twzGxSoUOj8WQ==" saltValue="905c+jUO58aUTtAhHe6Qyg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="J1:J2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 G1:G2 I1:I2 E1:E2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -19614,84 +19614,84 @@
       <c r="A1" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="82" t="s">
+      <c r="B1" s="84" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="83"/>
-      <c r="D1" s="83"/>
-      <c r="E1" s="83"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="94" t="s">
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="96" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="95"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="75" t="s">
+      <c r="H1" s="97"/>
+      <c r="I1" s="98"/>
+      <c r="J1" s="77" t="s">
         <v>180</v>
       </c>
-      <c r="K1" s="78" t="s">
+      <c r="K1" s="80" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="82" t="s">
+      <c r="L1" s="84" t="s">
         <v>94</v>
       </c>
-      <c r="M1" s="83"/>
-      <c r="N1" s="83"/>
-      <c r="O1" s="83"/>
-      <c r="P1" s="84"/>
+      <c r="M1" s="85"/>
+      <c r="N1" s="85"/>
+      <c r="O1" s="85"/>
+      <c r="P1" s="86"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
+      <c r="A2" s="83"/>
       <c r="B2" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="92" t="s">
+      <c r="C2" s="94" t="s">
         <v>178</v>
       </c>
       <c r="D2" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="87" t="s">
+      <c r="E2" s="89" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="93" t="s">
+      <c r="F2" s="95" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="89" t="s">
+      <c r="G2" s="91" t="s">
         <v>101</v>
       </c>
-      <c r="H2" s="90" t="s">
+      <c r="H2" s="92" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="97" t="s">
+      <c r="I2" s="75" t="s">
         <v>179</v>
       </c>
-      <c r="J2" s="76"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="85" t="s">
+      <c r="J2" s="78"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="87" t="s">
         <v>111</v>
       </c>
-      <c r="M2" s="85"/>
-      <c r="N2" s="85" t="s">
+      <c r="M2" s="87"/>
+      <c r="N2" s="87" t="s">
         <v>112</v>
       </c>
-      <c r="O2" s="85"/>
-      <c r="P2" s="86" t="s">
+      <c r="O2" s="87"/>
+      <c r="P2" s="88" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="70"/>
       <c r="B3" s="62"/>
-      <c r="C3" s="92"/>
+      <c r="C3" s="94"/>
       <c r="D3" s="62"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="93"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="91"/>
-      <c r="I3" s="98"/>
-      <c r="J3" s="77"/>
-      <c r="K3" s="80"/>
+      <c r="E3" s="90"/>
+      <c r="F3" s="95"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="93"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="79"/>
+      <c r="K3" s="82"/>
       <c r="L3" s="32" t="s">
         <v>3</v>
       </c>
@@ -19704,7 +19704,7 @@
       <c r="O3" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="P3" s="86"/>
+      <c r="P3" s="88"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -23309,6 +23309,7 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="Hbw1kM2GZdKiXn+tZ2jTENxb+s/WuKBOS35p7Hczzc8mzknealDwavQKvnmoI0NQ4e6Cl68C/s3alEC/HGJgTQ==" saltValue="phbtvlo1TeohYtjp0VwRjg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="G1:I1"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="K1:K3"/>
@@ -23325,7 +23326,6 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G1:I1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 O3 H2:H3 J1:K1" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -23373,23 +23373,23 @@
       <c r="A1" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="87" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85" t="s">
+      <c r="C1" s="87"/>
+      <c r="D1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="87"/>
+      <c r="G1" s="87" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
+      <c r="H1" s="87"/>
+      <c r="I1" s="87"/>
+      <c r="J1" s="87"/>
+      <c r="K1" s="87"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
+      <c r="A2" s="83"/>
       <c r="B2" s="65" t="s">
         <v>99</v>
       </c>
@@ -26163,14 +26163,14 @@
       <c r="AO1" s="74"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
-      <c r="B2" s="87" t="s">
+      <c r="A2" s="83"/>
+      <c r="B2" s="89" t="s">
         <v>181</v>
       </c>
       <c r="C2" s="100" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="75" t="s">
+      <c r="D2" s="77" t="s">
         <v>116</v>
       </c>
       <c r="E2" s="99" t="s">
@@ -26186,21 +26186,21 @@
       <c r="K2" s="101" t="s">
         <v>185</v>
       </c>
-      <c r="L2" s="93" t="s">
+      <c r="L2" s="95" t="s">
         <v>123</v>
       </c>
-      <c r="M2" s="93"/>
-      <c r="N2" s="93"/>
-      <c r="O2" s="93"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
+      <c r="O2" s="95"/>
       <c r="P2" s="99" t="s">
         <v>124</v>
       </c>
       <c r="Q2" s="99"/>
       <c r="R2" s="99"/>
-      <c r="S2" s="93" t="s">
+      <c r="S2" s="95" t="s">
         <v>22</v>
       </c>
-      <c r="T2" s="93"/>
+      <c r="T2" s="95"/>
       <c r="U2" s="99" t="s">
         <v>128</v>
       </c>
@@ -26240,28 +26240,28 @@
       <c r="AG2" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="AH2" s="93" t="s">
+      <c r="AH2" s="95" t="s">
         <v>138</v>
       </c>
-      <c r="AI2" s="93"/>
-      <c r="AJ2" s="93" t="s">
+      <c r="AI2" s="95"/>
+      <c r="AJ2" s="95" t="s">
         <v>139</v>
       </c>
-      <c r="AK2" s="93"/>
-      <c r="AL2" s="93" t="s">
+      <c r="AK2" s="95"/>
+      <c r="AL2" s="95" t="s">
         <v>140</v>
       </c>
-      <c r="AM2" s="93"/>
-      <c r="AN2" s="93" t="s">
+      <c r="AM2" s="95"/>
+      <c r="AN2" s="95" t="s">
         <v>141</v>
       </c>
-      <c r="AO2" s="93"/>
+      <c r="AO2" s="95"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A3" s="70"/>
-      <c r="B3" s="88"/>
+      <c r="B3" s="90"/>
       <c r="C3" s="67"/>
-      <c r="D3" s="77"/>
+      <c r="D3" s="79"/>
       <c r="E3" s="40" t="s">
         <v>20</v>
       </c>
@@ -34949,6 +34949,20 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="QMCtlxTdGMeqat8mqK+Cr1Fx43bg5wNSEIC6CaFaY0KIvb4EIpIjm6obel/9Z0Dv1oF2vEXJtDbPbO1sewkcAA==" saltValue="PmNUggfK+1j4qc6GrFpb8Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="X2:X3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -34965,20 +34979,6 @@
     <mergeCell ref="V2:V3"/>
     <mergeCell ref="AN2:AO2"/>
     <mergeCell ref="D2:D3"/>
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="X2:X3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN3 D2:D3 L3 M3 N3 O3 P3 Q3 R3 AH3 AI3 AJ3 AK3 AL3 AM3 AO3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -35043,55 +35043,55 @@
       <c r="L1" s="74"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
-      <c r="B2" s="93" t="s">
+      <c r="A2" s="83"/>
+      <c r="B2" s="95" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="93" t="s">
+      <c r="C2" s="95" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="93" t="s">
+      <c r="D2" s="95" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93" t="s">
+      <c r="E2" s="95"/>
+      <c r="F2" s="95"/>
+      <c r="G2" s="95"/>
+      <c r="H2" s="95" t="s">
         <v>146</v>
       </c>
-      <c r="I2" s="93"/>
-      <c r="J2" s="93"/>
-      <c r="K2" s="93"/>
-      <c r="L2" s="93" t="s">
+      <c r="I2" s="95"/>
+      <c r="J2" s="95"/>
+      <c r="K2" s="95"/>
+      <c r="L2" s="95" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="81"/>
-      <c r="B3" s="93"/>
-      <c r="C3" s="93"/>
-      <c r="D3" s="93" t="s">
+      <c r="A3" s="83"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="95" t="s">
         <v>188</v>
       </c>
-      <c r="E3" s="93"/>
-      <c r="F3" s="93" t="s">
+      <c r="E3" s="95"/>
+      <c r="F3" s="95" t="s">
         <v>189</v>
       </c>
-      <c r="G3" s="93"/>
-      <c r="H3" s="93" t="s">
+      <c r="G3" s="95"/>
+      <c r="H3" s="95" t="s">
         <v>148</v>
       </c>
-      <c r="I3" s="93"/>
-      <c r="J3" s="93" t="s">
+      <c r="I3" s="95"/>
+      <c r="J3" s="95" t="s">
         <v>147</v>
       </c>
-      <c r="K3" s="93"/>
-      <c r="L3" s="93"/>
+      <c r="K3" s="95"/>
+      <c r="L3" s="95"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="70"/>
-      <c r="B4" s="93"/>
-      <c r="C4" s="93"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="95"/>
       <c r="D4" s="46" t="s">
         <v>18</v>
       </c>
@@ -37981,22 +37981,22 @@
       <c r="F1" s="100" t="s">
         <v>150</v>
       </c>
-      <c r="G1" s="103"/>
-      <c r="H1" s="103"/>
-      <c r="I1" s="103"/>
-      <c r="J1" s="78" t="s">
+      <c r="G1" s="104"/>
+      <c r="H1" s="104"/>
+      <c r="I1" s="104"/>
+      <c r="J1" s="80" t="s">
         <v>77</v>
       </c>
-      <c r="K1" s="105" t="s">
+      <c r="K1" s="106" t="s">
         <v>155</v>
       </c>
-      <c r="L1" s="93" t="s">
+      <c r="L1" s="95" t="s">
         <v>65</v>
       </c>
-      <c r="M1" s="93" t="s">
+      <c r="M1" s="95" t="s">
         <v>66</v>
       </c>
-      <c r="N1" s="93" t="s">
+      <c r="N1" s="95" t="s">
         <v>67</v>
       </c>
       <c r="O1" s="72"/>
@@ -38006,18 +38006,18 @@
       <c r="Q1" s="74" t="s">
         <v>69</v>
       </c>
-      <c r="R1" s="93" t="s">
+      <c r="R1" s="95" t="s">
         <v>156</v>
       </c>
-      <c r="S1" s="93"/>
-      <c r="T1" s="93"/>
-      <c r="U1" s="93"/>
-      <c r="V1" s="93"/>
+      <c r="S1" s="95"/>
+      <c r="T1" s="95"/>
+      <c r="U1" s="95"/>
+      <c r="V1" s="95"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="106" t="s">
+      <c r="A2" s="83"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="103" t="s">
         <v>49</v>
       </c>
       <c r="D2" s="65" t="s">
@@ -38025,28 +38025,28 @@
       </c>
       <c r="E2" s="71"/>
       <c r="F2" s="67"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="104"/>
-      <c r="I2" s="104"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="105"/>
-      <c r="L2" s="93"/>
-      <c r="M2" s="93"/>
-      <c r="N2" s="93"/>
+      <c r="G2" s="105"/>
+      <c r="H2" s="105"/>
+      <c r="I2" s="105"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="106"/>
+      <c r="L2" s="95"/>
+      <c r="M2" s="95"/>
+      <c r="N2" s="95"/>
       <c r="O2" s="72"/>
-      <c r="P2" s="81"/>
+      <c r="P2" s="83"/>
       <c r="Q2" s="74"/>
       <c r="R2" s="99" t="s">
         <v>70</v>
       </c>
-      <c r="S2" s="93" t="s">
+      <c r="S2" s="95" t="s">
         <v>157</v>
       </c>
-      <c r="T2" s="93"/>
-      <c r="U2" s="93" t="s">
+      <c r="T2" s="95"/>
+      <c r="U2" s="95" t="s">
         <v>158</v>
       </c>
-      <c r="V2" s="93"/>
+      <c r="V2" s="95"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="70"/>
@@ -38070,10 +38070,10 @@
       <c r="I3" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="J3" s="80"/>
-      <c r="K3" s="105"/>
-      <c r="L3" s="93"/>
-      <c r="M3" s="93"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="106"/>
+      <c r="L3" s="95"/>
+      <c r="M3" s="95"/>
       <c r="N3" s="37" t="s">
         <v>71</v>
       </c>
@@ -42900,11 +42900,6 @@
   <sheetProtection algorithmName="SHA-512" hashValue="lB47MHjN7Q2DdsILtEIzmsVgF/RGH4fl4xMJSJCt+pfGM3g82GbEDtt7bi2H3b59LuCUpowHsRtb+ERWIIPhnQ==" saltValue="jdC1iYmDqqf8XUqPiuEltA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="17">
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
     <mergeCell ref="R1:V1"/>
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="S2:T2"/>
@@ -42917,6 +42912,11 @@
     <mergeCell ref="N1:O2"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="P1:P3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K3 I3 F3 G3 H3 U3 V3" xr:uid="{7CB5582D-4A36-46D9-AA38-ED8FA154223A}">
@@ -44617,14 +44617,14 @@
       <c r="C1" s="69" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="78" t="s">
+      <c r="D1" s="80" t="s">
         <v>161</v>
       </c>
       <c r="E1" s="107" t="s">
         <v>57</v>
       </c>
       <c r="F1" s="108"/>
-      <c r="G1" s="78" t="s">
+      <c r="G1" s="80" t="s">
         <v>163</v>
       </c>
       <c r="H1" s="69" t="s">
@@ -44640,14 +44640,14 @@
       <c r="A2" s="70"/>
       <c r="B2" s="70"/>
       <c r="C2" s="70"/>
-      <c r="D2" s="80"/>
+      <c r="D2" s="82"/>
       <c r="E2" s="39" t="s">
         <v>19</v>
       </c>
       <c r="F2" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="80"/>
+      <c r="G2" s="82"/>
       <c r="H2" s="70"/>
       <c r="I2" s="39" t="s">
         <v>164</v>

</xml_diff>

<commit_message>
Removal of a constraint in a cell
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\echassot\Desktop\repositories\data-reporting\iotc-reference-forms\form_reporting_templates\ros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCD133D-7224-4E04-93EA-25A03D08B21E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D5E3E8-453B-4A2C-AF46-C5CD0E8D6358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="c5/ou8Cml7ZkaDU47Tuu3WsAbYP19DC42wRzPBn3vsHWJE2MFn5j3m9vhk0UNMu/icNe5bym2Fttv6xJI1ZSAw==" workbookSaltValue="pG4NehU6lkQVWVHx3qNlvg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="5" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="879" activeTab="1" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -1133,6 +1133,27 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1187,23 +1208,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1236,9 +1251,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1278,18 +1290,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1301,9 +1301,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1313,6 +1310,9 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1666,24 +1666,24 @@
   <sheetData>
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="59" t="s">
         <v>95</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="54"/>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="E2" s="60"/>
+      <c r="F2" s="60"/>
+      <c r="G2" s="60"/>
+      <c r="H2" s="61"/>
     </row>
     <row r="3" spans="2:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="55"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="57"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="64"/>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="7"/>
@@ -1733,15 +1733,15 @@
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="13"/>
-      <c r="C8" s="58" t="s">
+      <c r="C8" s="65" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="58"/>
+      <c r="D8" s="65"/>
       <c r="E8" s="14"/>
-      <c r="F8" s="58" t="s">
+      <c r="F8" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="G8" s="58"/>
+      <c r="G8" s="65"/>
       <c r="H8" s="15"/>
     </row>
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
@@ -1923,11 +1923,11 @@
     </row>
     <row r="26" spans="2:8" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="13"/>
-      <c r="C26" s="59"/>
-      <c r="D26" s="60"/>
-      <c r="E26" s="60"/>
-      <c r="F26" s="60"/>
-      <c r="G26" s="61"/>
+      <c r="C26" s="66"/>
+      <c r="D26" s="67"/>
+      <c r="E26" s="67"/>
+      <c r="F26" s="67"/>
+      <c r="G26" s="68"/>
       <c r="H26" s="15"/>
     </row>
     <row r="27" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2012,15 +2012,15 @@
       <c r="D1" s="109" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="80" t="s">
+      <c r="E1" s="85" t="s">
         <v>163</v>
       </c>
-      <c r="F1" s="87" t="s">
+      <c r="F1" s="91" t="s">
         <v>169</v>
       </c>
-      <c r="G1" s="87"/>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
       <c r="J1" s="99" t="s">
         <v>170</v>
       </c>
@@ -2032,25 +2032,25 @@
       </c>
       <c r="O1" s="99"/>
       <c r="P1" s="99"/>
-      <c r="Q1" s="77" t="s">
+      <c r="Q1" s="82" t="s">
         <v>38</v>
       </c>
-      <c r="R1" s="72" t="s">
+      <c r="R1" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="S1" s="74"/>
-      <c r="T1" s="72" t="s">
+      <c r="S1" s="54"/>
+      <c r="T1" s="52" t="s">
         <v>168</v>
       </c>
-      <c r="U1" s="73"/>
-      <c r="V1" s="74"/>
+      <c r="U1" s="53"/>
+      <c r="V1" s="54"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="110"/>
       <c r="B2" s="110"/>
       <c r="C2" s="110"/>
       <c r="D2" s="110"/>
-      <c r="E2" s="82"/>
+      <c r="E2" s="87"/>
       <c r="F2" s="36" t="s">
         <v>19</v>
       </c>
@@ -2084,7 +2084,7 @@
       <c r="P2" s="45" t="s">
         <v>167</v>
       </c>
-      <c r="Q2" s="79"/>
+      <c r="Q2" s="84"/>
       <c r="R2" s="38" t="s">
         <v>53</v>
       </c>
@@ -6904,17 +6904,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="F0tc7B77v7QjLsOz0RLL7MWtNCPBw2o4Z9f2YID1JxL/5n/IHv5nh1k9azF4NV4h1VsWAZfQTfWlFcYB76PlMA==" saltValue="n01OBaL5NKfbkpK2LmYd9A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="Q1:Q2"/>
     <mergeCell ref="T1:V1"/>
     <mergeCell ref="R1:S1"/>
     <mergeCell ref="F1:I1"/>
     <mergeCell ref="J1:M1"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="N1:P1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="Q1:Q2"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E2 F2 H2 J2 L2 N2 Q1:Q2" xr:uid="{CF79E0B9-452F-42D7-82F9-4325C7CCE12E}">
@@ -6974,19 +6974,19 @@
       <c r="D1" s="109" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="77" t="s">
+      <c r="E1" s="82" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="77" t="s">
+      <c r="F1" s="82" t="s">
         <v>172</v>
       </c>
-      <c r="G1" s="77" t="s">
+      <c r="G1" s="82" t="s">
         <v>173</v>
       </c>
       <c r="H1" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="78" t="s">
+      <c r="I1" s="83" t="s">
         <v>174</v>
       </c>
       <c r="J1" s="111" t="s">
@@ -7001,13 +7001,13 @@
       <c r="B2" s="110"/>
       <c r="C2" s="110"/>
       <c r="D2" s="110"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="90"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="90"/>
-      <c r="K2" s="90"/>
+      <c r="E2" s="84"/>
+      <c r="F2" s="84"/>
+      <c r="G2" s="84"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="84"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="94"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
@@ -9612,17 +9612,17 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="7AjhL+fqXAsFucLZgoF2uPzgppBK+T/XTUzkX/JwpgqEiyXl3lYNCR44gk+4O6ySKgm58zlH7twzGxSoUOj8WQ==" saltValue="905c+jUO58aUTtAhHe6Qyg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="H1:H2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="I1:I2"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="G1:G2"/>
     <mergeCell ref="J1:J2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="H1:H2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F2 G1:G2 I1:I2 E1:E2" xr:uid="{D35AC15C-DF5E-4A91-9A87-73B80C6F3218}">
@@ -14192,117 +14192,117 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="69" t="s">
         <v>97</v>
       </c>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62" t="s">
+      <c r="C1" s="69"/>
+      <c r="D1" s="69" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62" t="s">
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="62"/>
-      <c r="T1" s="62"/>
-      <c r="U1" s="62"/>
-      <c r="V1" s="62"/>
-      <c r="W1" s="62"/>
-      <c r="X1" s="62"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
+      <c r="U1" s="69"/>
+      <c r="V1" s="69"/>
+      <c r="W1" s="69"/>
+      <c r="X1" s="69"/>
       <c r="Y1" s="4"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" s="62"/>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="65" t="s">
+      <c r="A2" s="69"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="72" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="71"/>
-      <c r="I2" s="65" t="s">
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="76"/>
+      <c r="I2" s="72" t="s">
         <v>47</v>
       </c>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="62"/>
-      <c r="X2" s="62"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="69"/>
+      <c r="V2" s="69"/>
+      <c r="W2" s="69"/>
+      <c r="X2" s="69"/>
       <c r="Y2" s="4"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="62"/>
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
-      <c r="D3" s="67" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="74" t="s">
         <v>99</v>
       </c>
-      <c r="E3" s="68"/>
-      <c r="F3" s="63" t="s">
+      <c r="E3" s="75"/>
+      <c r="F3" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="G3" s="64"/>
-      <c r="H3" s="69" t="s">
+      <c r="G3" s="71"/>
+      <c r="H3" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="I3" s="67" t="s">
+      <c r="I3" s="74" t="s">
         <v>99</v>
       </c>
-      <c r="J3" s="68"/>
-      <c r="K3" s="63" t="s">
+      <c r="J3" s="75"/>
+      <c r="K3" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="L3" s="64"/>
-      <c r="M3" s="69" t="s">
+      <c r="L3" s="71"/>
+      <c r="M3" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="N3" s="62" t="s">
+      <c r="N3" s="69" t="s">
         <v>103</v>
       </c>
-      <c r="O3" s="62"/>
-      <c r="P3" s="62" t="s">
+      <c r="O3" s="69"/>
+      <c r="P3" s="69" t="s">
         <v>104</v>
       </c>
-      <c r="Q3" s="62"/>
-      <c r="R3" s="62"/>
-      <c r="S3" s="62"/>
-      <c r="T3" s="62"/>
-      <c r="U3" s="72" t="s">
+      <c r="Q3" s="69"/>
+      <c r="R3" s="69"/>
+      <c r="S3" s="69"/>
+      <c r="T3" s="69"/>
+      <c r="U3" s="52" t="s">
         <v>105</v>
       </c>
-      <c r="V3" s="73"/>
-      <c r="W3" s="73"/>
-      <c r="X3" s="74"/>
+      <c r="V3" s="53"/>
+      <c r="W3" s="53"/>
+      <c r="X3" s="54"/>
     </row>
     <row r="4" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="62"/>
+      <c r="A4" s="69"/>
       <c r="B4" s="32" t="s">
         <v>79</v>
       </c>
@@ -14321,7 +14321,7 @@
       <c r="G4" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="70"/>
+      <c r="H4" s="57"/>
       <c r="I4" s="31" t="s">
         <v>101</v>
       </c>
@@ -14334,7 +14334,7 @@
       <c r="L4" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="M4" s="70"/>
+      <c r="M4" s="57"/>
       <c r="N4" s="32" t="s">
         <v>5</v>
       </c>
@@ -19546,7 +19546,7 @@
       <c r="X203" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="fVXWKxCR1qucAQa6utO/4fH1F9wUY8AODxxzlBRDtPgG4CCzIk4q2AsxwP756/R3QOL3Tba6UWhQjPmYXErNnw==" saltValue="wSFRtfCqKPzFlyH4k1jV2Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="46cFSM56bLsmreV25TOiQafDrffmltOeOr94Dy1gL5MIFPqeCQ/DibKgaNfsqxG+JnG4jGVm0+m2KMmbRCGwkA==" saltValue="GjrQooXRWNGpm6VKJS3d+A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="15">
     <mergeCell ref="A1:A4"/>
     <mergeCell ref="N3:O3"/>
@@ -19565,7 +19565,7 @@
     <mergeCell ref="U3:X3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5 W4 D4 E4 I4 J4 U4 V4 X4" xr:uid="{90961E5D-833B-4418-801E-6853BBBDB445}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X4 W4 D4 E4 I4 J4 U4 V4" xr:uid="{90961E5D-833B-4418-801E-6853BBBDB445}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19611,87 +19611,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="84" t="s">
+      <c r="B1" s="88" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="96" t="s">
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="97"/>
-      <c r="I1" s="98"/>
-      <c r="J1" s="77" t="s">
+      <c r="H1" s="78"/>
+      <c r="I1" s="79"/>
+      <c r="J1" s="82" t="s">
         <v>180</v>
       </c>
-      <c r="K1" s="80" t="s">
+      <c r="K1" s="85" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="84" t="s">
+      <c r="L1" s="88" t="s">
         <v>94</v>
       </c>
-      <c r="M1" s="85"/>
-      <c r="N1" s="85"/>
-      <c r="O1" s="85"/>
-      <c r="P1" s="86"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89"/>
+      <c r="P1" s="90"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="83"/>
-      <c r="B2" s="62" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="69" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="94" t="s">
+      <c r="C2" s="98" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="62" t="s">
+      <c r="D2" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="89" t="s">
+      <c r="E2" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="95" t="s">
+      <c r="F2" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="91" t="s">
+      <c r="G2" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="H2" s="92" t="s">
+      <c r="H2" s="96" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="75" t="s">
+      <c r="I2" s="80" t="s">
         <v>179</v>
       </c>
-      <c r="J2" s="78"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="87" t="s">
+      <c r="J2" s="83"/>
+      <c r="K2" s="86"/>
+      <c r="L2" s="91" t="s">
         <v>111</v>
       </c>
-      <c r="M2" s="87"/>
-      <c r="N2" s="87" t="s">
+      <c r="M2" s="91"/>
+      <c r="N2" s="91" t="s">
         <v>112</v>
       </c>
-      <c r="O2" s="87"/>
-      <c r="P2" s="88" t="s">
+      <c r="O2" s="91"/>
+      <c r="P2" s="92" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="62"/>
-      <c r="C3" s="94"/>
-      <c r="D3" s="62"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="91"/>
-      <c r="H3" s="93"/>
-      <c r="I3" s="76"/>
-      <c r="J3" s="79"/>
-      <c r="K3" s="82"/>
+      <c r="A3" s="57"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="98"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="94"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="95"/>
+      <c r="H3" s="97"/>
+      <c r="I3" s="81"/>
+      <c r="J3" s="84"/>
+      <c r="K3" s="87"/>
       <c r="L3" s="32" t="s">
         <v>3</v>
       </c>
@@ -19704,7 +19704,7 @@
       <c r="O3" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="P3" s="88"/>
+      <c r="P3" s="92"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -23309,11 +23309,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="Hbw1kM2GZdKiXn+tZ2jTENxb+s/WuKBOS35p7Hczzc8mzknealDwavQKvnmoI0NQ4e6Cl68C/s3alEC/HGJgTQ==" saltValue="phbtvlo1TeohYtjp0VwRjg==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="17">
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J1:J3"/>
-    <mergeCell ref="K1:K3"/>
-    <mergeCell ref="A1:A3"/>
     <mergeCell ref="L1:P1"/>
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="P2:P3"/>
@@ -23326,6 +23321,11 @@
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J1:J3"/>
+    <mergeCell ref="K1:K3"/>
+    <mergeCell ref="A1:A3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M3 O3 H2:H3 J1:K1" xr:uid="{ACED21EE-BC8F-4262-88C6-C5B6A4D7F4AF}">
@@ -23370,47 +23370,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="87" t="s">
+      <c r="B1" s="91" t="s">
         <v>114</v>
       </c>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87" t="s">
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91" t="s">
         <v>115</v>
       </c>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
-      <c r="J1" s="87"/>
-      <c r="K1" s="87"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="83"/>
-      <c r="B2" s="65" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="72" t="s">
         <v>99</v>
       </c>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="69" t="s">
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="55" t="s">
         <v>49</v>
       </c>
-      <c r="G2" s="65" t="s">
+      <c r="G2" s="72" t="s">
         <v>99</v>
       </c>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="69" t="s">
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="76"/>
+      <c r="K2" s="55" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
+      <c r="A3" s="57"/>
       <c r="B3" s="31" t="s">
         <v>101</v>
       </c>
@@ -23423,7 +23423,7 @@
       <c r="E3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="70"/>
+      <c r="F3" s="57"/>
       <c r="G3" s="31" t="s">
         <v>101</v>
       </c>
@@ -23436,7 +23436,7 @@
       <c r="J3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="K3" s="70"/>
+      <c r="K3" s="57"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -26112,65 +26112,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="72" t="s">
+      <c r="B1" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
-      <c r="N1" s="73"/>
-      <c r="O1" s="73"/>
-      <c r="P1" s="73"/>
-      <c r="Q1" s="73"/>
-      <c r="R1" s="73"/>
-      <c r="S1" s="73"/>
-      <c r="T1" s="74"/>
-      <c r="U1" s="72" t="s">
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="53"/>
+      <c r="P1" s="53"/>
+      <c r="Q1" s="53"/>
+      <c r="R1" s="53"/>
+      <c r="S1" s="53"/>
+      <c r="T1" s="54"/>
+      <c r="U1" s="52" t="s">
         <v>142</v>
       </c>
-      <c r="V1" s="73"/>
-      <c r="W1" s="73"/>
-      <c r="X1" s="73"/>
-      <c r="Y1" s="73"/>
-      <c r="Z1" s="73"/>
-      <c r="AA1" s="73"/>
-      <c r="AB1" s="73"/>
-      <c r="AC1" s="73"/>
-      <c r="AD1" s="73"/>
-      <c r="AE1" s="73"/>
-      <c r="AF1" s="73"/>
-      <c r="AG1" s="74"/>
-      <c r="AH1" s="72" t="s">
+      <c r="V1" s="53"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="53"/>
+      <c r="Y1" s="53"/>
+      <c r="Z1" s="53"/>
+      <c r="AA1" s="53"/>
+      <c r="AB1" s="53"/>
+      <c r="AC1" s="53"/>
+      <c r="AD1" s="53"/>
+      <c r="AE1" s="53"/>
+      <c r="AF1" s="53"/>
+      <c r="AG1" s="54"/>
+      <c r="AH1" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="AI1" s="73"/>
-      <c r="AJ1" s="73"/>
-      <c r="AK1" s="73"/>
-      <c r="AL1" s="73"/>
-      <c r="AM1" s="73"/>
-      <c r="AN1" s="73"/>
-      <c r="AO1" s="74"/>
+      <c r="AI1" s="53"/>
+      <c r="AJ1" s="53"/>
+      <c r="AK1" s="53"/>
+      <c r="AL1" s="53"/>
+      <c r="AM1" s="53"/>
+      <c r="AN1" s="53"/>
+      <c r="AO1" s="54"/>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A2" s="83"/>
-      <c r="B2" s="89" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="93" t="s">
         <v>181</v>
       </c>
       <c r="C2" s="100" t="s">
         <v>182</v>
       </c>
-      <c r="D2" s="77" t="s">
+      <c r="D2" s="82" t="s">
         <v>116</v>
       </c>
       <c r="E2" s="99" t="s">
@@ -26186,21 +26186,21 @@
       <c r="K2" s="101" t="s">
         <v>185</v>
       </c>
-      <c r="L2" s="95" t="s">
+      <c r="L2" s="58" t="s">
         <v>123</v>
       </c>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="95"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="58"/>
       <c r="P2" s="99" t="s">
         <v>124</v>
       </c>
       <c r="Q2" s="99"/>
       <c r="R2" s="99"/>
-      <c r="S2" s="95" t="s">
+      <c r="S2" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="T2" s="95"/>
+      <c r="T2" s="58"/>
       <c r="U2" s="99" t="s">
         <v>128</v>
       </c>
@@ -26240,28 +26240,28 @@
       <c r="AG2" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="AH2" s="95" t="s">
+      <c r="AH2" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="AI2" s="95"/>
-      <c r="AJ2" s="95" t="s">
+      <c r="AI2" s="58"/>
+      <c r="AJ2" s="58" t="s">
         <v>139</v>
       </c>
-      <c r="AK2" s="95"/>
-      <c r="AL2" s="95" t="s">
+      <c r="AK2" s="58"/>
+      <c r="AL2" s="58" t="s">
         <v>140</v>
       </c>
-      <c r="AM2" s="95"/>
-      <c r="AN2" s="95" t="s">
+      <c r="AM2" s="58"/>
+      <c r="AN2" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="AO2" s="95"/>
+      <c r="AO2" s="58"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="67"/>
-      <c r="D3" s="79"/>
+      <c r="A3" s="57"/>
+      <c r="B3" s="94"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="84"/>
       <c r="E3" s="40" t="s">
         <v>20</v>
       </c>
@@ -34949,20 +34949,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="QMCtlxTdGMeqat8mqK+Cr1Fx43bg5wNSEIC6CaFaY0KIvb4EIpIjm6obel/9Z0Dv1oF2vEXJtDbPbO1sewkcAA==" saltValue="PmNUggfK+1j4qc6GrFpb8Q==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="30">
-    <mergeCell ref="AC2:AC3"/>
-    <mergeCell ref="AG2:AG3"/>
-    <mergeCell ref="L2:O2"/>
-    <mergeCell ref="AL2:AM2"/>
-    <mergeCell ref="AH2:AI2"/>
-    <mergeCell ref="AJ2:AK2"/>
-    <mergeCell ref="AF2:AF3"/>
-    <mergeCell ref="AE2:AE3"/>
-    <mergeCell ref="AD2:AD3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="Z2:Z3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="X2:X3"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:T1"/>
     <mergeCell ref="U1:AG1"/>
@@ -34979,6 +34965,20 @@
     <mergeCell ref="V2:V3"/>
     <mergeCell ref="AN2:AO2"/>
     <mergeCell ref="D2:D3"/>
+    <mergeCell ref="AC2:AC3"/>
+    <mergeCell ref="AG2:AG3"/>
+    <mergeCell ref="L2:O2"/>
+    <mergeCell ref="AL2:AM2"/>
+    <mergeCell ref="AH2:AI2"/>
+    <mergeCell ref="AJ2:AK2"/>
+    <mergeCell ref="AF2:AF3"/>
+    <mergeCell ref="AE2:AE3"/>
+    <mergeCell ref="AD2:AD3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="X2:X3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AN3 D2:D3 L3 M3 N3 O3 P3 Q3 R3 AH3 AI3 AJ3 AK3 AL3 AM3 AO3" xr:uid="{7AE1CE56-A690-401C-B311-F5FE2246C553}">
@@ -35023,75 +35023,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="72" t="s">
+      <c r="B1" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="C1" s="74"/>
-      <c r="D1" s="72" t="s">
+      <c r="C1" s="54"/>
+      <c r="D1" s="52" t="s">
         <v>145</v>
       </c>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="74"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="54"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="83"/>
-      <c r="B2" s="95" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="58" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="95" t="s">
+      <c r="C2" s="58" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="95" t="s">
+      <c r="D2" s="58" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95" t="s">
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95" t="s">
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+      <c r="L2" s="58" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="83"/>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95" t="s">
+      <c r="A3" s="56"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58" t="s">
         <v>188</v>
       </c>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95" t="s">
+      <c r="E3" s="58"/>
+      <c r="F3" s="58" t="s">
         <v>189</v>
       </c>
-      <c r="G3" s="95"/>
-      <c r="H3" s="95" t="s">
+      <c r="G3" s="58"/>
+      <c r="H3" s="58" t="s">
         <v>148</v>
       </c>
-      <c r="I3" s="95"/>
-      <c r="J3" s="95" t="s">
+      <c r="I3" s="58"/>
+      <c r="J3" s="58" t="s">
         <v>147</v>
       </c>
-      <c r="K3" s="95"/>
-      <c r="L3" s="95"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="70"/>
-      <c r="B4" s="95"/>
-      <c r="C4" s="95"/>
+      <c r="A4" s="57"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
       <c r="D4" s="46" t="s">
         <v>18</v>
       </c>
@@ -37967,91 +37967,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="69" t="s">
+      <c r="B1" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="65" t="s">
+      <c r="C1" s="72" t="s">
         <v>149</v>
       </c>
-      <c r="D1" s="66"/>
-      <c r="E1" s="71"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="76"/>
       <c r="F1" s="100" t="s">
         <v>150</v>
       </c>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="104"/>
-      <c r="J1" s="80" t="s">
+      <c r="G1" s="103"/>
+      <c r="H1" s="103"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="85" t="s">
         <v>77</v>
       </c>
-      <c r="K1" s="106" t="s">
+      <c r="K1" s="105" t="s">
         <v>155</v>
       </c>
-      <c r="L1" s="95" t="s">
+      <c r="L1" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="M1" s="95" t="s">
+      <c r="M1" s="58" t="s">
         <v>66</v>
       </c>
-      <c r="N1" s="95" t="s">
+      <c r="N1" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="O1" s="72"/>
-      <c r="P1" s="69" t="s">
+      <c r="O1" s="52"/>
+      <c r="P1" s="55" t="s">
         <v>68</v>
       </c>
-      <c r="Q1" s="74" t="s">
+      <c r="Q1" s="54" t="s">
         <v>69</v>
       </c>
-      <c r="R1" s="95" t="s">
+      <c r="R1" s="58" t="s">
         <v>156</v>
       </c>
-      <c r="S1" s="95"/>
-      <c r="T1" s="95"/>
-      <c r="U1" s="95"/>
-      <c r="V1" s="95"/>
+      <c r="S1" s="58"/>
+      <c r="T1" s="58"/>
+      <c r="U1" s="58"/>
+      <c r="V1" s="58"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A2" s="83"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="103" t="s">
+      <c r="A2" s="56"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="106" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="65" t="s">
+      <c r="D2" s="72" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="71"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="105"/>
-      <c r="H2" s="105"/>
-      <c r="I2" s="105"/>
-      <c r="J2" s="81"/>
-      <c r="K2" s="106"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="95"/>
-      <c r="N2" s="95"/>
-      <c r="O2" s="72"/>
-      <c r="P2" s="83"/>
-      <c r="Q2" s="74"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="104"/>
+      <c r="J2" s="86"/>
+      <c r="K2" s="105"/>
+      <c r="L2" s="58"/>
+      <c r="M2" s="58"/>
+      <c r="N2" s="58"/>
+      <c r="O2" s="52"/>
+      <c r="P2" s="56"/>
+      <c r="Q2" s="54"/>
       <c r="R2" s="99" t="s">
         <v>70</v>
       </c>
-      <c r="S2" s="95" t="s">
+      <c r="S2" s="58" t="s">
         <v>157</v>
       </c>
-      <c r="T2" s="95"/>
-      <c r="U2" s="95" t="s">
+      <c r="T2" s="58"/>
+      <c r="U2" s="58" t="s">
         <v>158</v>
       </c>
-      <c r="V2" s="95"/>
+      <c r="V2" s="58"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="70"/>
-      <c r="C3" s="63"/>
+      <c r="A3" s="57"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="70"/>
       <c r="D3" s="32" t="s">
         <v>0</v>
       </c>
@@ -38070,18 +38070,18 @@
       <c r="I3" s="44" t="s">
         <v>154</v>
       </c>
-      <c r="J3" s="82"/>
-      <c r="K3" s="106"/>
-      <c r="L3" s="95"/>
-      <c r="M3" s="95"/>
+      <c r="J3" s="87"/>
+      <c r="K3" s="105"/>
+      <c r="L3" s="58"/>
+      <c r="M3" s="58"/>
       <c r="N3" s="37" t="s">
         <v>71</v>
       </c>
       <c r="O3" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="P3" s="70"/>
-      <c r="Q3" s="74"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="54"/>
       <c r="R3" s="99"/>
       <c r="S3" s="40" t="s">
         <v>73</v>
@@ -42900,6 +42900,11 @@
   <sheetProtection algorithmName="SHA-512" hashValue="lB47MHjN7Q2DdsILtEIzmsVgF/RGH4fl4xMJSJCt+pfGM3g82GbEDtt7bi2H3b59LuCUpowHsRtb+ERWIIPhnQ==" saltValue="jdC1iYmDqqf8XUqPiuEltA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="17">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
     <mergeCell ref="R1:V1"/>
     <mergeCell ref="R2:R3"/>
     <mergeCell ref="S2:T2"/>
@@ -42912,11 +42917,6 @@
     <mergeCell ref="N1:O2"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="P1:P3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K1:K3 I3 F3 G3 H3 U3 V3" xr:uid="{7CB5582D-4A36-46D9-AA38-ED8FA154223A}">
@@ -44608,47 +44608,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="69" t="s">
+      <c r="A1" s="55" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="69" t="s">
+      <c r="B1" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="69" t="s">
+      <c r="C1" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="80" t="s">
+      <c r="D1" s="85" t="s">
         <v>161</v>
       </c>
       <c r="E1" s="107" t="s">
         <v>57</v>
       </c>
       <c r="F1" s="108"/>
-      <c r="G1" s="80" t="s">
+      <c r="G1" s="85" t="s">
         <v>163</v>
       </c>
-      <c r="H1" s="69" t="s">
+      <c r="H1" s="55" t="s">
         <v>162</v>
       </c>
-      <c r="I1" s="65" t="s">
+      <c r="I1" s="72" t="s">
         <v>35</v>
       </c>
-      <c r="J1" s="66"/>
-      <c r="K1" s="71"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="76"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="82"/>
+      <c r="A2" s="57"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="87"/>
       <c r="E2" s="39" t="s">
         <v>19</v>
       </c>
       <c r="F2" s="39" t="s">
         <v>56</v>
       </c>
-      <c r="G2" s="82"/>
-      <c r="H2" s="70"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="57"/>
       <c r="I2" s="39" t="s">
         <v>164</v>
       </c>

</xml_diff>

<commit_message>
logical response code lists added to setting and cetacean setting
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C112324-41FB-0F46-A14C-06EE8319A6DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BE1425F-552F-254F-8F23-79F1C7BC3743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="c5/ou8Cml7ZkaDU47Tuu3WsAbYP19DC42wRzPBn3vsHWJE2MFn5j3m9vhk0UNMu/icNe5bym2Fttv6xJI1ZSAw==" workbookSaltValue="pG4NehU6lkQVWVHx3qNlvg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16360" tabRatio="879" firstSheet="1" activeTab="5" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16360" tabRatio="879" firstSheet="1" activeTab="7" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -994,7 +994,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
@@ -1324,6 +1324,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -38097,10 +38103,10 @@
       <c r="P3" s="70"/>
       <c r="Q3" s="74"/>
       <c r="R3" s="99"/>
-      <c r="S3" s="39" t="s">
+      <c r="S3" s="114" t="s">
         <v>73</v>
       </c>
-      <c r="T3" s="39" t="s">
+      <c r="T3" s="114" t="s">
         <v>74</v>
       </c>
       <c r="U3" s="33" t="s">
@@ -42911,7 +42917,7 @@
       <c r="V203" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="SUEhtek1xjdHrbhxzS10tklKE6LDK3INEq0x/apGRQZ4wd8qhkNkaK2pjf/Dc5DheFyyovwYwOOIRWqRZcbsIA==" saltValue="mUomoVIUflQXJbTqgskr3A==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="LGbLE0X4mphbrvyDB8iHZbZ5jGyiClFuG1okIajSb/6AE438B82i1uIvOTrWorRsJspA6UxPow4rvWi+AhQlIA==" saltValue="1ksA3tQoetcJpOHsQN0vtA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="17">
     <mergeCell ref="C2:C3"/>
@@ -42946,6 +42952,8 @@
     <hyperlink ref="V3" r:id="rId6" location="FADtailDesigns" xr:uid="{4EC548E9-585E-4A0F-8A11-B2D8DE7871DC}"/>
     <hyperlink ref="U3" r:id="rId7" location="FADraftDesigns" xr:uid="{56C6FE4F-AE5D-4D49-879C-6D4A0BF75DFF}"/>
     <hyperlink ref="J1:J3" r:id="rId8" location="schoolTypeCategories" display="SCHOOL_TYPES" xr:uid="{8EC575CB-432D-43D0-8C91-3FACD4044FFB}"/>
+    <hyperlink ref="S3" r:id="rId9" location="logicalResponses" xr:uid="{860C6C50-4466-3940-9B0A-F8CB030221D5}"/>
+    <hyperlink ref="T3" r:id="rId10" location="logicalResponses" xr:uid="{02ADBEB1-CD08-E74C-96CC-90C58B333795}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -42974,7 +42982,7 @@
       <c r="B1" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="115" t="s">
         <v>75</v>
       </c>
       <c r="D1" s="35" t="s">
@@ -42983,7 +42991,7 @@
       <c r="E1" s="31" t="s">
         <v>186</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="115" t="s">
         <v>76</v>
       </c>
     </row>
@@ -44588,7 +44596,7 @@
       <c r="F201" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="G6ZwYN709Jy1AWIWQxAxVplHZP5uP/NiiAIMHJ1doR9/7pTBWAVy2vieUW0vMIWYxyRbT7D7xiLCv9S3N8yYaQ==" saltValue="uuk0pmAMVaL17oFOYQ/XcQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="UhrGzLwIH2JWpEZUUgcwvaPIu5FPGaxVInDJYWlNOKBbqTKmKl6F4H6+z/aTMLMuHNoEgABRFAKIxGa5DhkC5g==" saltValue="AG5AZvp511RQ1Xg2O8UwZA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1" xr:uid="{9A958104-A80B-4B1E-AB96-42BA504F7B3D}">
       <formula1>"&lt;0&gt;0"</formula1>
@@ -44596,6 +44604,8 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D1" r:id="rId1" location="cetaceansAndWhaleSharks" xr:uid="{F9440529-0B3C-4E2C-9C30-02C136FF531F}"/>
+    <hyperlink ref="C1" r:id="rId2" location="logicalResponses" xr:uid="{45E8DB2A-EC4B-CE4E-8A5C-271AA5DE39FD}"/>
+    <hyperlink ref="F1" r:id="rId3" location="logicalResponses" xr:uid="{0CA90A9C-0AC7-474C-A06E-8C6556CA9097}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
"straight" fields removed from specimen details
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BE1425F-552F-254F-8F23-79F1C7BC3743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF7B744-D3EA-9342-9A98-97FC8850D4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="c5/ou8Cml7ZkaDU47Tuu3WsAbYP19DC42wRzPBn3vsHWJE2MFn5j3m9vhk0UNMu/icNe5bym2Fttv6xJI1ZSAw==" workbookSaltValue="pG4NehU6lkQVWVHx3qNlvg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16360" tabRatio="879" firstSheet="1" activeTab="7" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16360" tabRatio="879" firstSheet="1" activeTab="9" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="194">
   <si>
     <t>LATITUDE</t>
   </si>
@@ -184,9 +184,6 @@
   </si>
   <si>
     <t>PHOTO_ID</t>
-  </si>
-  <si>
-    <t>IS_STRAIGHT</t>
   </si>
   <si>
     <t>EMBARKATION</t>
@@ -1670,7 +1667,7 @@
     <row r="1" spans="2:8" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B2" s="52" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="53"/>
       <c r="D2" s="53"/>
@@ -1691,14 +1688,14 @@
     <row r="4" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G4" s="11">
         <v>5</v>
@@ -1717,7 +1714,7 @@
     <row r="6" spans="2:8" ht="19" x14ac:dyDescent="0.25">
       <c r="B6" s="13"/>
       <c r="C6" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
@@ -1737,12 +1734,12 @@
     <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B8" s="13"/>
       <c r="C8" s="58" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D8" s="58"/>
       <c r="E8" s="14"/>
       <c r="F8" s="58" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G8" s="58"/>
       <c r="H8" s="15"/>
@@ -1750,12 +1747,12 @@
     <row r="9" spans="2:8" ht="45" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="13"/>
       <c r="C9" s="17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D9" s="18"/>
       <c r="E9" s="14"/>
       <c r="F9" s="17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G9" s="18"/>
       <c r="H9" s="15"/>
@@ -1763,12 +1760,12 @@
     <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" s="13"/>
       <c r="C10" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D10" s="18"/>
       <c r="E10" s="14"/>
       <c r="F10" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G10" s="18"/>
       <c r="H10" s="15"/>
@@ -1785,7 +1782,7 @@
     <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" s="13"/>
       <c r="C12" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D12" s="21"/>
       <c r="E12" s="14"/>
@@ -1796,7 +1793,7 @@
     <row r="13" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B13" s="13"/>
       <c r="C13" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D13" s="21"/>
       <c r="E13" s="14"/>
@@ -1825,7 +1822,7 @@
     <row r="16" spans="2:8" ht="19" x14ac:dyDescent="0.25">
       <c r="B16" s="13"/>
       <c r="C16" s="16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
@@ -1845,7 +1842,7 @@
     <row r="18" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B18" s="13"/>
       <c r="C18" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="14"/>
@@ -1856,7 +1853,7 @@
     <row r="19" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B19" s="13"/>
       <c r="C19" s="51" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D19" s="23"/>
       <c r="E19" s="14"/>
@@ -1867,7 +1864,7 @@
     <row r="20" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B20" s="13"/>
       <c r="C20" s="51" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D20" s="23"/>
       <c r="E20" s="14"/>
@@ -1878,7 +1875,7 @@
     <row r="21" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B21" s="13"/>
       <c r="C21" s="51" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D21" s="23"/>
       <c r="E21" s="14"/>
@@ -1907,7 +1904,7 @@
     <row r="24" spans="2:8" ht="19" x14ac:dyDescent="0.25">
       <c r="B24" s="13"/>
       <c r="C24" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D24" s="20"/>
       <c r="E24" s="14"/>
@@ -1975,7 +1972,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:V202"/>
+  <dimension ref="A1:T202"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.33203125" style="3" bestFit="1" customWidth="1"/>
@@ -1986,69 +1983,65 @@
     <col min="6" max="6" width="11" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="22.5" style="3" customWidth="1"/>
-    <col min="9" max="9" width="14.5" style="3" customWidth="1"/>
-    <col min="10" max="10" width="11" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="23.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5" style="3" customWidth="1"/>
-    <col min="14" max="14" width="19.33203125" style="3" customWidth="1"/>
-    <col min="15" max="15" width="12.5" style="3" customWidth="1"/>
-    <col min="16" max="16" width="34.5" style="3" customWidth="1"/>
-    <col min="17" max="17" width="9.1640625" style="3"/>
-    <col min="18" max="18" width="16.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.6640625" style="3" customWidth="1"/>
-    <col min="20" max="20" width="11" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="23.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="23.5" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="23.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.33203125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="12.5" style="3" customWidth="1"/>
+    <col min="14" max="14" width="34.5" style="3" customWidth="1"/>
+    <col min="15" max="15" width="9.1640625" style="3"/>
+    <col min="16" max="16" width="16.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.6640625" style="3" customWidth="1"/>
+    <col min="18" max="18" width="11" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A1" s="109" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="109" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="109" t="s">
+      <c r="C1" s="109" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="D1" s="109" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="109" t="s">
-        <v>61</v>
-      </c>
       <c r="E1" s="96" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F1" s="79" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G1" s="79"/>
       <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="99" t="s">
-        <v>170</v>
+      <c r="I1" s="99" t="s">
+        <v>169</v>
       </c>
+      <c r="J1" s="99"/>
       <c r="K1" s="99"/>
-      <c r="L1" s="99"/>
-      <c r="M1" s="99"/>
-      <c r="N1" s="99" t="s">
+      <c r="L1" s="99" t="s">
         <v>35</v>
       </c>
-      <c r="O1" s="99"/>
-      <c r="P1" s="99"/>
-      <c r="Q1" s="93" t="s">
+      <c r="M1" s="99"/>
+      <c r="N1" s="99"/>
+      <c r="O1" s="93" t="s">
         <v>38</v>
       </c>
+      <c r="P1" s="72" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" s="74"/>
       <c r="R1" s="72" t="s">
-        <v>55</v>
+        <v>167</v>
       </c>
-      <c r="S1" s="74"/>
-      <c r="T1" s="72" t="s">
-        <v>168</v>
-      </c>
-      <c r="U1" s="73"/>
-      <c r="V1" s="74"/>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="S1" s="73"/>
+      <c r="T1" s="74"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A2" s="110"/>
       <c r="B2" s="110"/>
       <c r="C2" s="110"/>
@@ -2061,50 +2054,44 @@
         <v>37</v>
       </c>
       <c r="H2" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="I2" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="L2" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="M2" s="34" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="44" t="s">
         <v>166</v>
       </c>
-      <c r="I2" s="31" t="s">
-        <v>45</v>
+      <c r="O2" s="95"/>
+      <c r="P2" s="37" t="s">
+        <v>52</v>
       </c>
-      <c r="J2" s="30" t="s">
+      <c r="Q2" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="R2" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="34" t="s">
-        <v>37</v>
-      </c>
-      <c r="L2" s="30" t="s">
-        <v>166</v>
-      </c>
-      <c r="M2" s="34" t="s">
-        <v>45</v>
-      </c>
-      <c r="N2" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="O2" s="34" t="s">
-        <v>36</v>
-      </c>
-      <c r="P2" s="44" t="s">
-        <v>167</v>
-      </c>
-      <c r="Q2" s="95"/>
-      <c r="R2" s="37" t="s">
-        <v>53</v>
-      </c>
-      <c r="S2" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="T2" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="U2" s="44" t="s">
+      <c r="S2" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="V2" s="34" t="s">
-        <v>187</v>
+      <c r="T2" s="34" t="s">
+        <v>186</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -2125,10 +2112,8 @@
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2149,10 +2134,8 @@
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -2173,10 +2156,8 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -2197,10 +2178,8 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2221,10 +2200,8 @@
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2245,10 +2222,8 @@
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -2269,10 +2244,8 @@
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
       <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2293,10 +2266,8 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
       <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -2317,10 +2288,8 @@
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2341,10 +2310,8 @@
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
       <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="2"/>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -2365,10 +2332,8 @@
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -2389,10 +2354,8 @@
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
       <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2413,10 +2376,8 @@
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
       <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -2437,10 +2398,8 @@
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="2"/>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -2461,10 +2420,8 @@
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -2485,10 +2442,8 @@
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
-      <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -2509,10 +2464,8 @@
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
       <c r="T19" s="2"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="2"/>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -2533,10 +2486,8 @@
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
       <c r="T20" s="2"/>
-      <c r="U20" s="2"/>
-      <c r="V20" s="2"/>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -2557,10 +2508,8 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
       <c r="T21" s="2"/>
-      <c r="U21" s="2"/>
-      <c r="V21" s="2"/>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -2581,10 +2530,8 @@
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
       <c r="T22" s="2"/>
-      <c r="U22" s="2"/>
-      <c r="V22" s="2"/>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -2605,10 +2552,8 @@
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
       <c r="T23" s="2"/>
-      <c r="U23" s="2"/>
-      <c r="V23" s="2"/>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -2629,10 +2574,8 @@
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
       <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-      <c r="V24" s="2"/>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -2653,10 +2596,8 @@
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
-      <c r="U25" s="2"/>
-      <c r="V25" s="2"/>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -2677,10 +2618,8 @@
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
       <c r="T26" s="2"/>
-      <c r="U26" s="2"/>
-      <c r="V26" s="2"/>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -2701,10 +2640,8 @@
       <c r="R27" s="2"/>
       <c r="S27" s="2"/>
       <c r="T27" s="2"/>
-      <c r="U27" s="2"/>
-      <c r="V27" s="2"/>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -2725,10 +2662,8 @@
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
-      <c r="U28" s="2"/>
-      <c r="V28" s="2"/>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -2749,10 +2684,8 @@
       <c r="R29" s="2"/>
       <c r="S29" s="2"/>
       <c r="T29" s="2"/>
-      <c r="U29" s="2"/>
-      <c r="V29" s="2"/>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -2773,10 +2706,8 @@
       <c r="R30" s="2"/>
       <c r="S30" s="2"/>
       <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -2797,10 +2728,8 @@
       <c r="R31" s="2"/>
       <c r="S31" s="2"/>
       <c r="T31" s="2"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="2"/>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -2821,10 +2750,8 @@
       <c r="R32" s="2"/>
       <c r="S32" s="2"/>
       <c r="T32" s="2"/>
-      <c r="U32" s="2"/>
-      <c r="V32" s="2"/>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -2845,10 +2772,8 @@
       <c r="R33" s="2"/>
       <c r="S33" s="2"/>
       <c r="T33" s="2"/>
-      <c r="U33" s="2"/>
-      <c r="V33" s="2"/>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -2869,10 +2794,8 @@
       <c r="R34" s="2"/>
       <c r="S34" s="2"/>
       <c r="T34" s="2"/>
-      <c r="U34" s="2"/>
-      <c r="V34" s="2"/>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -2893,10 +2816,8 @@
       <c r="R35" s="2"/>
       <c r="S35" s="2"/>
       <c r="T35" s="2"/>
-      <c r="U35" s="2"/>
-      <c r="V35" s="2"/>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -2917,10 +2838,8 @@
       <c r="R36" s="2"/>
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
-      <c r="U36" s="2"/>
-      <c r="V36" s="2"/>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -2941,10 +2860,8 @@
       <c r="R37" s="2"/>
       <c r="S37" s="2"/>
       <c r="T37" s="2"/>
-      <c r="U37" s="2"/>
-      <c r="V37" s="2"/>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>
@@ -2965,10 +2882,8 @@
       <c r="R38" s="2"/>
       <c r="S38" s="2"/>
       <c r="T38" s="2"/>
-      <c r="U38" s="2"/>
-      <c r="V38" s="2"/>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -2989,10 +2904,8 @@
       <c r="R39" s="2"/>
       <c r="S39" s="2"/>
       <c r="T39" s="2"/>
-      <c r="U39" s="2"/>
-      <c r="V39" s="2"/>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
@@ -3013,10 +2926,8 @@
       <c r="R40" s="2"/>
       <c r="S40" s="2"/>
       <c r="T40" s="2"/>
-      <c r="U40" s="2"/>
-      <c r="V40" s="2"/>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -3037,10 +2948,8 @@
       <c r="R41" s="2"/>
       <c r="S41" s="2"/>
       <c r="T41" s="2"/>
-      <c r="U41" s="2"/>
-      <c r="V41" s="2"/>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
@@ -3061,10 +2970,8 @@
       <c r="R42" s="2"/>
       <c r="S42" s="2"/>
       <c r="T42" s="2"/>
-      <c r="U42" s="2"/>
-      <c r="V42" s="2"/>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -3085,10 +2992,8 @@
       <c r="R43" s="2"/>
       <c r="S43" s="2"/>
       <c r="T43" s="2"/>
-      <c r="U43" s="2"/>
-      <c r="V43" s="2"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
       <c r="B44" s="2"/>
       <c r="C44" s="2"/>
@@ -3109,10 +3014,8 @@
       <c r="R44" s="2"/>
       <c r="S44" s="2"/>
       <c r="T44" s="2"/>
-      <c r="U44" s="2"/>
-      <c r="V44" s="2"/>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -3133,10 +3036,8 @@
       <c r="R45" s="2"/>
       <c r="S45" s="2"/>
       <c r="T45" s="2"/>
-      <c r="U45" s="2"/>
-      <c r="V45" s="2"/>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
@@ -3157,10 +3058,8 @@
       <c r="R46" s="2"/>
       <c r="S46" s="2"/>
       <c r="T46" s="2"/>
-      <c r="U46" s="2"/>
-      <c r="V46" s="2"/>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -3181,10 +3080,8 @@
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
       <c r="T47" s="2"/>
-      <c r="U47" s="2"/>
-      <c r="V47" s="2"/>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -3205,10 +3102,8 @@
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
       <c r="T48" s="2"/>
-      <c r="U48" s="2"/>
-      <c r="V48" s="2"/>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -3229,10 +3124,8 @@
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
       <c r="T49" s="2"/>
-      <c r="U49" s="2"/>
-      <c r="V49" s="2"/>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -3253,10 +3146,8 @@
       <c r="R50" s="2"/>
       <c r="S50" s="2"/>
       <c r="T50" s="2"/>
-      <c r="U50" s="2"/>
-      <c r="V50" s="2"/>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -3277,10 +3168,8 @@
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
       <c r="T51" s="2"/>
-      <c r="U51" s="2"/>
-      <c r="V51" s="2"/>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -3301,10 +3190,8 @@
       <c r="R52" s="2"/>
       <c r="S52" s="2"/>
       <c r="T52" s="2"/>
-      <c r="U52" s="2"/>
-      <c r="V52" s="2"/>
-    </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -3325,10 +3212,8 @@
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
       <c r="T53" s="2"/>
-      <c r="U53" s="2"/>
-      <c r="V53" s="2"/>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -3349,10 +3234,8 @@
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
       <c r="T54" s="2"/>
-      <c r="U54" s="2"/>
-      <c r="V54" s="2"/>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -3373,10 +3256,8 @@
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
       <c r="T55" s="2"/>
-      <c r="U55" s="2"/>
-      <c r="V55" s="2"/>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -3397,10 +3278,8 @@
       <c r="R56" s="2"/>
       <c r="S56" s="2"/>
       <c r="T56" s="2"/>
-      <c r="U56" s="2"/>
-      <c r="V56" s="2"/>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -3421,10 +3300,8 @@
       <c r="R57" s="2"/>
       <c r="S57" s="2"/>
       <c r="T57" s="2"/>
-      <c r="U57" s="2"/>
-      <c r="V57" s="2"/>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -3445,10 +3322,8 @@
       <c r="R58" s="2"/>
       <c r="S58" s="2"/>
       <c r="T58" s="2"/>
-      <c r="U58" s="2"/>
-      <c r="V58" s="2"/>
-    </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -3469,10 +3344,8 @@
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
       <c r="T59" s="2"/>
-      <c r="U59" s="2"/>
-      <c r="V59" s="2"/>
-    </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -3493,10 +3366,8 @@
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
       <c r="T60" s="2"/>
-      <c r="U60" s="2"/>
-      <c r="V60" s="2"/>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -3517,10 +3388,8 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
       <c r="T61" s="2"/>
-      <c r="U61" s="2"/>
-      <c r="V61" s="2"/>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -3541,10 +3410,8 @@
       <c r="R62" s="2"/>
       <c r="S62" s="2"/>
       <c r="T62" s="2"/>
-      <c r="U62" s="2"/>
-      <c r="V62" s="2"/>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -3565,10 +3432,8 @@
       <c r="R63" s="2"/>
       <c r="S63" s="2"/>
       <c r="T63" s="2"/>
-      <c r="U63" s="2"/>
-      <c r="V63" s="2"/>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -3589,10 +3454,8 @@
       <c r="R64" s="2"/>
       <c r="S64" s="2"/>
       <c r="T64" s="2"/>
-      <c r="U64" s="2"/>
-      <c r="V64" s="2"/>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -3613,10 +3476,8 @@
       <c r="R65" s="2"/>
       <c r="S65" s="2"/>
       <c r="T65" s="2"/>
-      <c r="U65" s="2"/>
-      <c r="V65" s="2"/>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
@@ -3637,10 +3498,8 @@
       <c r="R66" s="2"/>
       <c r="S66" s="2"/>
       <c r="T66" s="2"/>
-      <c r="U66" s="2"/>
-      <c r="V66" s="2"/>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -3661,10 +3520,8 @@
       <c r="R67" s="2"/>
       <c r="S67" s="2"/>
       <c r="T67" s="2"/>
-      <c r="U67" s="2"/>
-      <c r="V67" s="2"/>
-    </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
@@ -3685,10 +3542,8 @@
       <c r="R68" s="2"/>
       <c r="S68" s="2"/>
       <c r="T68" s="2"/>
-      <c r="U68" s="2"/>
-      <c r="V68" s="2"/>
-    </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -3709,10 +3564,8 @@
       <c r="R69" s="2"/>
       <c r="S69" s="2"/>
       <c r="T69" s="2"/>
-      <c r="U69" s="2"/>
-      <c r="V69" s="2"/>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2"/>
@@ -3733,10 +3586,8 @@
       <c r="R70" s="2"/>
       <c r="S70" s="2"/>
       <c r="T70" s="2"/>
-      <c r="U70" s="2"/>
-      <c r="V70" s="2"/>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -3757,10 +3608,8 @@
       <c r="R71" s="2"/>
       <c r="S71" s="2"/>
       <c r="T71" s="2"/>
-      <c r="U71" s="2"/>
-      <c r="V71" s="2"/>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
       <c r="C72" s="2"/>
@@ -3781,10 +3630,8 @@
       <c r="R72" s="2"/>
       <c r="S72" s="2"/>
       <c r="T72" s="2"/>
-      <c r="U72" s="2"/>
-      <c r="V72" s="2"/>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -3805,10 +3652,8 @@
       <c r="R73" s="2"/>
       <c r="S73" s="2"/>
       <c r="T73" s="2"/>
-      <c r="U73" s="2"/>
-      <c r="V73" s="2"/>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="2"/>
@@ -3829,10 +3674,8 @@
       <c r="R74" s="2"/>
       <c r="S74" s="2"/>
       <c r="T74" s="2"/>
-      <c r="U74" s="2"/>
-      <c r="V74" s="2"/>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -3853,10 +3696,8 @@
       <c r="R75" s="2"/>
       <c r="S75" s="2"/>
       <c r="T75" s="2"/>
-      <c r="U75" s="2"/>
-      <c r="V75" s="2"/>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
@@ -3877,10 +3718,8 @@
       <c r="R76" s="2"/>
       <c r="S76" s="2"/>
       <c r="T76" s="2"/>
-      <c r="U76" s="2"/>
-      <c r="V76" s="2"/>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -3901,10 +3740,8 @@
       <c r="R77" s="2"/>
       <c r="S77" s="2"/>
       <c r="T77" s="2"/>
-      <c r="U77" s="2"/>
-      <c r="V77" s="2"/>
-    </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
@@ -3925,10 +3762,8 @@
       <c r="R78" s="2"/>
       <c r="S78" s="2"/>
       <c r="T78" s="2"/>
-      <c r="U78" s="2"/>
-      <c r="V78" s="2"/>
-    </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -3949,10 +3784,8 @@
       <c r="R79" s="2"/>
       <c r="S79" s="2"/>
       <c r="T79" s="2"/>
-      <c r="U79" s="2"/>
-      <c r="V79" s="2"/>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
@@ -3973,10 +3806,8 @@
       <c r="R80" s="2"/>
       <c r="S80" s="2"/>
       <c r="T80" s="2"/>
-      <c r="U80" s="2"/>
-      <c r="V80" s="2"/>
-    </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -3997,10 +3828,8 @@
       <c r="R81" s="2"/>
       <c r="S81" s="2"/>
       <c r="T81" s="2"/>
-      <c r="U81" s="2"/>
-      <c r="V81" s="2"/>
-    </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="82" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
@@ -4021,10 +3850,8 @@
       <c r="R82" s="2"/>
       <c r="S82" s="2"/>
       <c r="T82" s="2"/>
-      <c r="U82" s="2"/>
-      <c r="V82" s="2"/>
-    </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="83" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -4045,10 +3872,8 @@
       <c r="R83" s="2"/>
       <c r="S83" s="2"/>
       <c r="T83" s="2"/>
-      <c r="U83" s="2"/>
-      <c r="V83" s="2"/>
-    </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
@@ -4069,10 +3894,8 @@
       <c r="R84" s="2"/>
       <c r="S84" s="2"/>
       <c r="T84" s="2"/>
-      <c r="U84" s="2"/>
-      <c r="V84" s="2"/>
-    </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="85" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -4093,10 +3916,8 @@
       <c r="R85" s="2"/>
       <c r="S85" s="2"/>
       <c r="T85" s="2"/>
-      <c r="U85" s="2"/>
-      <c r="V85" s="2"/>
-    </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="86" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
       <c r="B86" s="2"/>
       <c r="C86" s="2"/>
@@ -4117,10 +3938,8 @@
       <c r="R86" s="2"/>
       <c r="S86" s="2"/>
       <c r="T86" s="2"/>
-      <c r="U86" s="2"/>
-      <c r="V86" s="2"/>
-    </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="87" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -4141,10 +3960,8 @@
       <c r="R87" s="2"/>
       <c r="S87" s="2"/>
       <c r="T87" s="2"/>
-      <c r="U87" s="2"/>
-      <c r="V87" s="2"/>
-    </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="88" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
@@ -4165,10 +3982,8 @@
       <c r="R88" s="2"/>
       <c r="S88" s="2"/>
       <c r="T88" s="2"/>
-      <c r="U88" s="2"/>
-      <c r="V88" s="2"/>
-    </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="89" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -4189,10 +4004,8 @@
       <c r="R89" s="2"/>
       <c r="S89" s="2"/>
       <c r="T89" s="2"/>
-      <c r="U89" s="2"/>
-      <c r="V89" s="2"/>
-    </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="90" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
@@ -4213,10 +4026,8 @@
       <c r="R90" s="2"/>
       <c r="S90" s="2"/>
       <c r="T90" s="2"/>
-      <c r="U90" s="2"/>
-      <c r="V90" s="2"/>
-    </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="91" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -4237,10 +4048,8 @@
       <c r="R91" s="2"/>
       <c r="S91" s="2"/>
       <c r="T91" s="2"/>
-      <c r="U91" s="2"/>
-      <c r="V91" s="2"/>
-    </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="92" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
       <c r="B92" s="2"/>
       <c r="C92" s="2"/>
@@ -4261,10 +4070,8 @@
       <c r="R92" s="2"/>
       <c r="S92" s="2"/>
       <c r="T92" s="2"/>
-      <c r="U92" s="2"/>
-      <c r="V92" s="2"/>
-    </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="93" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -4285,10 +4092,8 @@
       <c r="R93" s="2"/>
       <c r="S93" s="2"/>
       <c r="T93" s="2"/>
-      <c r="U93" s="2"/>
-      <c r="V93" s="2"/>
-    </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="94" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
       <c r="B94" s="2"/>
       <c r="C94" s="2"/>
@@ -4309,10 +4114,8 @@
       <c r="R94" s="2"/>
       <c r="S94" s="2"/>
       <c r="T94" s="2"/>
-      <c r="U94" s="2"/>
-      <c r="V94" s="2"/>
-    </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="95" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -4333,10 +4136,8 @@
       <c r="R95" s="2"/>
       <c r="S95" s="2"/>
       <c r="T95" s="2"/>
-      <c r="U95" s="2"/>
-      <c r="V95" s="2"/>
-    </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="96" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
       <c r="B96" s="2"/>
       <c r="C96" s="2"/>
@@ -4357,10 +4158,8 @@
       <c r="R96" s="2"/>
       <c r="S96" s="2"/>
       <c r="T96" s="2"/>
-      <c r="U96" s="2"/>
-      <c r="V96" s="2"/>
-    </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -4381,10 +4180,8 @@
       <c r="R97" s="2"/>
       <c r="S97" s="2"/>
       <c r="T97" s="2"/>
-      <c r="U97" s="2"/>
-      <c r="V97" s="2"/>
-    </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -4405,10 +4202,8 @@
       <c r="R98" s="2"/>
       <c r="S98" s="2"/>
       <c r="T98" s="2"/>
-      <c r="U98" s="2"/>
-      <c r="V98" s="2"/>
-    </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -4429,10 +4224,8 @@
       <c r="R99" s="2"/>
       <c r="S99" s="2"/>
       <c r="T99" s="2"/>
-      <c r="U99" s="2"/>
-      <c r="V99" s="2"/>
-    </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -4453,10 +4246,8 @@
       <c r="R100" s="2"/>
       <c r="S100" s="2"/>
       <c r="T100" s="2"/>
-      <c r="U100" s="2"/>
-      <c r="V100" s="2"/>
-    </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="101" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -4477,10 +4268,8 @@
       <c r="R101" s="2"/>
       <c r="S101" s="2"/>
       <c r="T101" s="2"/>
-      <c r="U101" s="2"/>
-      <c r="V101" s="2"/>
-    </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -4501,10 +4290,8 @@
       <c r="R102" s="2"/>
       <c r="S102" s="2"/>
       <c r="T102" s="2"/>
-      <c r="U102" s="2"/>
-      <c r="V102" s="2"/>
-    </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -4525,10 +4312,8 @@
       <c r="R103" s="2"/>
       <c r="S103" s="2"/>
       <c r="T103" s="2"/>
-      <c r="U103" s="2"/>
-      <c r="V103" s="2"/>
-    </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -4549,10 +4334,8 @@
       <c r="R104" s="2"/>
       <c r="S104" s="2"/>
       <c r="T104" s="2"/>
-      <c r="U104" s="2"/>
-      <c r="V104" s="2"/>
-    </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
@@ -4573,10 +4356,8 @@
       <c r="R105" s="2"/>
       <c r="S105" s="2"/>
       <c r="T105" s="2"/>
-      <c r="U105" s="2"/>
-      <c r="V105" s="2"/>
-    </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -4597,10 +4378,8 @@
       <c r="R106" s="2"/>
       <c r="S106" s="2"/>
       <c r="T106" s="2"/>
-      <c r="U106" s="2"/>
-      <c r="V106" s="2"/>
-    </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -4621,10 +4400,8 @@
       <c r="R107" s="2"/>
       <c r="S107" s="2"/>
       <c r="T107" s="2"/>
-      <c r="U107" s="2"/>
-      <c r="V107" s="2"/>
-    </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
@@ -4645,10 +4422,8 @@
       <c r="R108" s="2"/>
       <c r="S108" s="2"/>
       <c r="T108" s="2"/>
-      <c r="U108" s="2"/>
-      <c r="V108" s="2"/>
-    </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
@@ -4669,10 +4444,8 @@
       <c r="R109" s="2"/>
       <c r="S109" s="2"/>
       <c r="T109" s="2"/>
-      <c r="U109" s="2"/>
-      <c r="V109" s="2"/>
-    </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
@@ -4693,10 +4466,8 @@
       <c r="R110" s="2"/>
       <c r="S110" s="2"/>
       <c r="T110" s="2"/>
-      <c r="U110" s="2"/>
-      <c r="V110" s="2"/>
-    </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="111" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
@@ -4717,10 +4488,8 @@
       <c r="R111" s="2"/>
       <c r="S111" s="2"/>
       <c r="T111" s="2"/>
-      <c r="U111" s="2"/>
-      <c r="V111" s="2"/>
-    </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="112" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
@@ -4741,10 +4510,8 @@
       <c r="R112" s="2"/>
       <c r="S112" s="2"/>
       <c r="T112" s="2"/>
-      <c r="U112" s="2"/>
-      <c r="V112" s="2"/>
-    </row>
-    <row r="113" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
@@ -4765,10 +4532,8 @@
       <c r="R113" s="2"/>
       <c r="S113" s="2"/>
       <c r="T113" s="2"/>
-      <c r="U113" s="2"/>
-      <c r="V113" s="2"/>
-    </row>
-    <row r="114" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="114" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
@@ -4789,10 +4554,8 @@
       <c r="R114" s="2"/>
       <c r="S114" s="2"/>
       <c r="T114" s="2"/>
-      <c r="U114" s="2"/>
-      <c r="V114" s="2"/>
-    </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
@@ -4813,10 +4576,8 @@
       <c r="R115" s="2"/>
       <c r="S115" s="2"/>
       <c r="T115" s="2"/>
-      <c r="U115" s="2"/>
-      <c r="V115" s="2"/>
-    </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A116" s="2"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
@@ -4837,10 +4598,8 @@
       <c r="R116" s="2"/>
       <c r="S116" s="2"/>
       <c r="T116" s="2"/>
-      <c r="U116" s="2"/>
-      <c r="V116" s="2"/>
-    </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
@@ -4861,10 +4620,8 @@
       <c r="R117" s="2"/>
       <c r="S117" s="2"/>
       <c r="T117" s="2"/>
-      <c r="U117" s="2"/>
-      <c r="V117" s="2"/>
-    </row>
-    <row r="118" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A118" s="2"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
@@ -4885,10 +4642,8 @@
       <c r="R118" s="2"/>
       <c r="S118" s="2"/>
       <c r="T118" s="2"/>
-      <c r="U118" s="2"/>
-      <c r="V118" s="2"/>
-    </row>
-    <row r="119" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="119" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A119" s="2"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
@@ -4909,10 +4664,8 @@
       <c r="R119" s="2"/>
       <c r="S119" s="2"/>
       <c r="T119" s="2"/>
-      <c r="U119" s="2"/>
-      <c r="V119" s="2"/>
-    </row>
-    <row r="120" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="120" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
@@ -4933,10 +4686,8 @@
       <c r="R120" s="2"/>
       <c r="S120" s="2"/>
       <c r="T120" s="2"/>
-      <c r="U120" s="2"/>
-      <c r="V120" s="2"/>
-    </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A121" s="2"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
@@ -4957,10 +4708,8 @@
       <c r="R121" s="2"/>
       <c r="S121" s="2"/>
       <c r="T121" s="2"/>
-      <c r="U121" s="2"/>
-      <c r="V121" s="2"/>
-    </row>
-    <row r="122" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A122" s="2"/>
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
@@ -4981,10 +4730,8 @@
       <c r="R122" s="2"/>
       <c r="S122" s="2"/>
       <c r="T122" s="2"/>
-      <c r="U122" s="2"/>
-      <c r="V122" s="2"/>
-    </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A123" s="2"/>
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
@@ -5005,10 +4752,8 @@
       <c r="R123" s="2"/>
       <c r="S123" s="2"/>
       <c r="T123" s="2"/>
-      <c r="U123" s="2"/>
-      <c r="V123" s="2"/>
-    </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A124" s="2"/>
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
@@ -5029,10 +4774,8 @@
       <c r="R124" s="2"/>
       <c r="S124" s="2"/>
       <c r="T124" s="2"/>
-      <c r="U124" s="2"/>
-      <c r="V124" s="2"/>
-    </row>
-    <row r="125" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="125" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A125" s="2"/>
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
@@ -5053,10 +4796,8 @@
       <c r="R125" s="2"/>
       <c r="S125" s="2"/>
       <c r="T125" s="2"/>
-      <c r="U125" s="2"/>
-      <c r="V125" s="2"/>
-    </row>
-    <row r="126" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="126" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A126" s="2"/>
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
@@ -5077,10 +4818,8 @@
       <c r="R126" s="2"/>
       <c r="S126" s="2"/>
       <c r="T126" s="2"/>
-      <c r="U126" s="2"/>
-      <c r="V126" s="2"/>
-    </row>
-    <row r="127" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="127" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A127" s="2"/>
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
@@ -5101,10 +4840,8 @@
       <c r="R127" s="2"/>
       <c r="S127" s="2"/>
       <c r="T127" s="2"/>
-      <c r="U127" s="2"/>
-      <c r="V127" s="2"/>
-    </row>
-    <row r="128" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="128" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A128" s="2"/>
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
@@ -5125,10 +4862,8 @@
       <c r="R128" s="2"/>
       <c r="S128" s="2"/>
       <c r="T128" s="2"/>
-      <c r="U128" s="2"/>
-      <c r="V128" s="2"/>
-    </row>
-    <row r="129" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="129" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A129" s="2"/>
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
@@ -5149,10 +4884,8 @@
       <c r="R129" s="2"/>
       <c r="S129" s="2"/>
       <c r="T129" s="2"/>
-      <c r="U129" s="2"/>
-      <c r="V129" s="2"/>
-    </row>
-    <row r="130" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="130" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A130" s="2"/>
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
@@ -5173,10 +4906,8 @@
       <c r="R130" s="2"/>
       <c r="S130" s="2"/>
       <c r="T130" s="2"/>
-      <c r="U130" s="2"/>
-      <c r="V130" s="2"/>
-    </row>
-    <row r="131" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="131" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A131" s="2"/>
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
@@ -5197,10 +4928,8 @@
       <c r="R131" s="2"/>
       <c r="S131" s="2"/>
       <c r="T131" s="2"/>
-      <c r="U131" s="2"/>
-      <c r="V131" s="2"/>
-    </row>
-    <row r="132" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="132" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A132" s="2"/>
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
@@ -5221,10 +4950,8 @@
       <c r="R132" s="2"/>
       <c r="S132" s="2"/>
       <c r="T132" s="2"/>
-      <c r="U132" s="2"/>
-      <c r="V132" s="2"/>
-    </row>
-    <row r="133" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="133" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A133" s="2"/>
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
@@ -5245,10 +4972,8 @@
       <c r="R133" s="2"/>
       <c r="S133" s="2"/>
       <c r="T133" s="2"/>
-      <c r="U133" s="2"/>
-      <c r="V133" s="2"/>
-    </row>
-    <row r="134" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="134" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A134" s="2"/>
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
@@ -5269,10 +4994,8 @@
       <c r="R134" s="2"/>
       <c r="S134" s="2"/>
       <c r="T134" s="2"/>
-      <c r="U134" s="2"/>
-      <c r="V134" s="2"/>
-    </row>
-    <row r="135" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="135" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A135" s="2"/>
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
@@ -5293,10 +5016,8 @@
       <c r="R135" s="2"/>
       <c r="S135" s="2"/>
       <c r="T135" s="2"/>
-      <c r="U135" s="2"/>
-      <c r="V135" s="2"/>
-    </row>
-    <row r="136" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="136" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A136" s="2"/>
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
@@ -5317,10 +5038,8 @@
       <c r="R136" s="2"/>
       <c r="S136" s="2"/>
       <c r="T136" s="2"/>
-      <c r="U136" s="2"/>
-      <c r="V136" s="2"/>
-    </row>
-    <row r="137" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="137" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A137" s="2"/>
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
@@ -5341,10 +5060,8 @@
       <c r="R137" s="2"/>
       <c r="S137" s="2"/>
       <c r="T137" s="2"/>
-      <c r="U137" s="2"/>
-      <c r="V137" s="2"/>
-    </row>
-    <row r="138" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="138" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A138" s="2"/>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
@@ -5365,10 +5082,8 @@
       <c r="R138" s="2"/>
       <c r="S138" s="2"/>
       <c r="T138" s="2"/>
-      <c r="U138" s="2"/>
-      <c r="V138" s="2"/>
-    </row>
-    <row r="139" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="139" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A139" s="2"/>
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
@@ -5389,10 +5104,8 @@
       <c r="R139" s="2"/>
       <c r="S139" s="2"/>
       <c r="T139" s="2"/>
-      <c r="U139" s="2"/>
-      <c r="V139" s="2"/>
-    </row>
-    <row r="140" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="140" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A140" s="2"/>
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
@@ -5413,10 +5126,8 @@
       <c r="R140" s="2"/>
       <c r="S140" s="2"/>
       <c r="T140" s="2"/>
-      <c r="U140" s="2"/>
-      <c r="V140" s="2"/>
-    </row>
-    <row r="141" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="141" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A141" s="2"/>
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
@@ -5437,10 +5148,8 @@
       <c r="R141" s="2"/>
       <c r="S141" s="2"/>
       <c r="T141" s="2"/>
-      <c r="U141" s="2"/>
-      <c r="V141" s="2"/>
-    </row>
-    <row r="142" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="142" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A142" s="2"/>
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
@@ -5461,10 +5170,8 @@
       <c r="R142" s="2"/>
       <c r="S142" s="2"/>
       <c r="T142" s="2"/>
-      <c r="U142" s="2"/>
-      <c r="V142" s="2"/>
-    </row>
-    <row r="143" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="143" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A143" s="2"/>
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
@@ -5485,10 +5192,8 @@
       <c r="R143" s="2"/>
       <c r="S143" s="2"/>
       <c r="T143" s="2"/>
-      <c r="U143" s="2"/>
-      <c r="V143" s="2"/>
-    </row>
-    <row r="144" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="144" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A144" s="2"/>
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
@@ -5509,10 +5214,8 @@
       <c r="R144" s="2"/>
       <c r="S144" s="2"/>
       <c r="T144" s="2"/>
-      <c r="U144" s="2"/>
-      <c r="V144" s="2"/>
-    </row>
-    <row r="145" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="145" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -5533,10 +5236,8 @@
       <c r="R145" s="2"/>
       <c r="S145" s="2"/>
       <c r="T145" s="2"/>
-      <c r="U145" s="2"/>
-      <c r="V145" s="2"/>
-    </row>
-    <row r="146" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="146" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
@@ -5557,10 +5258,8 @@
       <c r="R146" s="2"/>
       <c r="S146" s="2"/>
       <c r="T146" s="2"/>
-      <c r="U146" s="2"/>
-      <c r="V146" s="2"/>
-    </row>
-    <row r="147" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="147" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -5581,10 +5280,8 @@
       <c r="R147" s="2"/>
       <c r="S147" s="2"/>
       <c r="T147" s="2"/>
-      <c r="U147" s="2"/>
-      <c r="V147" s="2"/>
-    </row>
-    <row r="148" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="148" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
@@ -5605,10 +5302,8 @@
       <c r="R148" s="2"/>
       <c r="S148" s="2"/>
       <c r="T148" s="2"/>
-      <c r="U148" s="2"/>
-      <c r="V148" s="2"/>
-    </row>
-    <row r="149" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="149" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -5629,10 +5324,8 @@
       <c r="R149" s="2"/>
       <c r="S149" s="2"/>
       <c r="T149" s="2"/>
-      <c r="U149" s="2"/>
-      <c r="V149" s="2"/>
-    </row>
-    <row r="150" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="150" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
@@ -5653,10 +5346,8 @@
       <c r="R150" s="2"/>
       <c r="S150" s="2"/>
       <c r="T150" s="2"/>
-      <c r="U150" s="2"/>
-      <c r="V150" s="2"/>
-    </row>
-    <row r="151" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="151" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -5677,10 +5368,8 @@
       <c r="R151" s="2"/>
       <c r="S151" s="2"/>
       <c r="T151" s="2"/>
-      <c r="U151" s="2"/>
-      <c r="V151" s="2"/>
-    </row>
-    <row r="152" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="152" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
@@ -5701,10 +5390,8 @@
       <c r="R152" s="2"/>
       <c r="S152" s="2"/>
       <c r="T152" s="2"/>
-      <c r="U152" s="2"/>
-      <c r="V152" s="2"/>
-    </row>
-    <row r="153" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="153" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -5725,10 +5412,8 @@
       <c r="R153" s="2"/>
       <c r="S153" s="2"/>
       <c r="T153" s="2"/>
-      <c r="U153" s="2"/>
-      <c r="V153" s="2"/>
-    </row>
-    <row r="154" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="154" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
@@ -5749,10 +5434,8 @@
       <c r="R154" s="2"/>
       <c r="S154" s="2"/>
       <c r="T154" s="2"/>
-      <c r="U154" s="2"/>
-      <c r="V154" s="2"/>
-    </row>
-    <row r="155" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="155" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
@@ -5773,10 +5456,8 @@
       <c r="R155" s="2"/>
       <c r="S155" s="2"/>
       <c r="T155" s="2"/>
-      <c r="U155" s="2"/>
-      <c r="V155" s="2"/>
-    </row>
-    <row r="156" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="156" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
@@ -5797,10 +5478,8 @@
       <c r="R156" s="2"/>
       <c r="S156" s="2"/>
       <c r="T156" s="2"/>
-      <c r="U156" s="2"/>
-      <c r="V156" s="2"/>
-    </row>
-    <row r="157" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="157" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
@@ -5821,10 +5500,8 @@
       <c r="R157" s="2"/>
       <c r="S157" s="2"/>
       <c r="T157" s="2"/>
-      <c r="U157" s="2"/>
-      <c r="V157" s="2"/>
-    </row>
-    <row r="158" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="158" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
@@ -5845,10 +5522,8 @@
       <c r="R158" s="2"/>
       <c r="S158" s="2"/>
       <c r="T158" s="2"/>
-      <c r="U158" s="2"/>
-      <c r="V158" s="2"/>
-    </row>
-    <row r="159" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="159" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
@@ -5869,10 +5544,8 @@
       <c r="R159" s="2"/>
       <c r="S159" s="2"/>
       <c r="T159" s="2"/>
-      <c r="U159" s="2"/>
-      <c r="V159" s="2"/>
-    </row>
-    <row r="160" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="160" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
@@ -5893,10 +5566,8 @@
       <c r="R160" s="2"/>
       <c r="S160" s="2"/>
       <c r="T160" s="2"/>
-      <c r="U160" s="2"/>
-      <c r="V160" s="2"/>
-    </row>
-    <row r="161" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="161" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A161" s="2"/>
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
@@ -5917,10 +5588,8 @@
       <c r="R161" s="2"/>
       <c r="S161" s="2"/>
       <c r="T161" s="2"/>
-      <c r="U161" s="2"/>
-      <c r="V161" s="2"/>
-    </row>
-    <row r="162" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="162" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A162" s="2"/>
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
@@ -5941,10 +5610,8 @@
       <c r="R162" s="2"/>
       <c r="S162" s="2"/>
       <c r="T162" s="2"/>
-      <c r="U162" s="2"/>
-      <c r="V162" s="2"/>
-    </row>
-    <row r="163" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="163" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A163" s="2"/>
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
@@ -5965,10 +5632,8 @@
       <c r="R163" s="2"/>
       <c r="S163" s="2"/>
       <c r="T163" s="2"/>
-      <c r="U163" s="2"/>
-      <c r="V163" s="2"/>
-    </row>
-    <row r="164" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="164" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A164" s="2"/>
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
@@ -5989,10 +5654,8 @@
       <c r="R164" s="2"/>
       <c r="S164" s="2"/>
       <c r="T164" s="2"/>
-      <c r="U164" s="2"/>
-      <c r="V164" s="2"/>
-    </row>
-    <row r="165" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="165" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A165" s="2"/>
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
@@ -6013,10 +5676,8 @@
       <c r="R165" s="2"/>
       <c r="S165" s="2"/>
       <c r="T165" s="2"/>
-      <c r="U165" s="2"/>
-      <c r="V165" s="2"/>
-    </row>
-    <row r="166" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="166" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A166" s="2"/>
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
@@ -6037,10 +5698,8 @@
       <c r="R166" s="2"/>
       <c r="S166" s="2"/>
       <c r="T166" s="2"/>
-      <c r="U166" s="2"/>
-      <c r="V166" s="2"/>
-    </row>
-    <row r="167" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="167" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A167" s="2"/>
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
@@ -6061,10 +5720,8 @@
       <c r="R167" s="2"/>
       <c r="S167" s="2"/>
       <c r="T167" s="2"/>
-      <c r="U167" s="2"/>
-      <c r="V167" s="2"/>
-    </row>
-    <row r="168" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="168" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A168" s="2"/>
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
@@ -6085,10 +5742,8 @@
       <c r="R168" s="2"/>
       <c r="S168" s="2"/>
       <c r="T168" s="2"/>
-      <c r="U168" s="2"/>
-      <c r="V168" s="2"/>
-    </row>
-    <row r="169" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="169" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A169" s="2"/>
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
@@ -6109,10 +5764,8 @@
       <c r="R169" s="2"/>
       <c r="S169" s="2"/>
       <c r="T169" s="2"/>
-      <c r="U169" s="2"/>
-      <c r="V169" s="2"/>
-    </row>
-    <row r="170" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="170" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A170" s="2"/>
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
@@ -6133,10 +5786,8 @@
       <c r="R170" s="2"/>
       <c r="S170" s="2"/>
       <c r="T170" s="2"/>
-      <c r="U170" s="2"/>
-      <c r="V170" s="2"/>
-    </row>
-    <row r="171" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="171" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A171" s="2"/>
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
@@ -6157,10 +5808,8 @@
       <c r="R171" s="2"/>
       <c r="S171" s="2"/>
       <c r="T171" s="2"/>
-      <c r="U171" s="2"/>
-      <c r="V171" s="2"/>
-    </row>
-    <row r="172" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="172" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A172" s="2"/>
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
@@ -6181,10 +5830,8 @@
       <c r="R172" s="2"/>
       <c r="S172" s="2"/>
       <c r="T172" s="2"/>
-      <c r="U172" s="2"/>
-      <c r="V172" s="2"/>
-    </row>
-    <row r="173" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="173" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A173" s="2"/>
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
@@ -6205,10 +5852,8 @@
       <c r="R173" s="2"/>
       <c r="S173" s="2"/>
       <c r="T173" s="2"/>
-      <c r="U173" s="2"/>
-      <c r="V173" s="2"/>
-    </row>
-    <row r="174" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="174" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A174" s="2"/>
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
@@ -6229,10 +5874,8 @@
       <c r="R174" s="2"/>
       <c r="S174" s="2"/>
       <c r="T174" s="2"/>
-      <c r="U174" s="2"/>
-      <c r="V174" s="2"/>
-    </row>
-    <row r="175" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="175" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A175" s="2"/>
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
@@ -6253,10 +5896,8 @@
       <c r="R175" s="2"/>
       <c r="S175" s="2"/>
       <c r="T175" s="2"/>
-      <c r="U175" s="2"/>
-      <c r="V175" s="2"/>
-    </row>
-    <row r="176" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="176" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A176" s="2"/>
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
@@ -6277,10 +5918,8 @@
       <c r="R176" s="2"/>
       <c r="S176" s="2"/>
       <c r="T176" s="2"/>
-      <c r="U176" s="2"/>
-      <c r="V176" s="2"/>
-    </row>
-    <row r="177" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="177" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A177" s="2"/>
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
@@ -6301,10 +5940,8 @@
       <c r="R177" s="2"/>
       <c r="S177" s="2"/>
       <c r="T177" s="2"/>
-      <c r="U177" s="2"/>
-      <c r="V177" s="2"/>
-    </row>
-    <row r="178" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="178" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A178" s="2"/>
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
@@ -6325,10 +5962,8 @@
       <c r="R178" s="2"/>
       <c r="S178" s="2"/>
       <c r="T178" s="2"/>
-      <c r="U178" s="2"/>
-      <c r="V178" s="2"/>
-    </row>
-    <row r="179" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="179" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A179" s="2"/>
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
@@ -6349,10 +5984,8 @@
       <c r="R179" s="2"/>
       <c r="S179" s="2"/>
       <c r="T179" s="2"/>
-      <c r="U179" s="2"/>
-      <c r="V179" s="2"/>
-    </row>
-    <row r="180" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="180" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A180" s="2"/>
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
@@ -6373,10 +6006,8 @@
       <c r="R180" s="2"/>
       <c r="S180" s="2"/>
       <c r="T180" s="2"/>
-      <c r="U180" s="2"/>
-      <c r="V180" s="2"/>
-    </row>
-    <row r="181" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="181" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A181" s="2"/>
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
@@ -6397,10 +6028,8 @@
       <c r="R181" s="2"/>
       <c r="S181" s="2"/>
       <c r="T181" s="2"/>
-      <c r="U181" s="2"/>
-      <c r="V181" s="2"/>
-    </row>
-    <row r="182" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="182" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A182" s="2"/>
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
@@ -6421,10 +6050,8 @@
       <c r="R182" s="2"/>
       <c r="S182" s="2"/>
       <c r="T182" s="2"/>
-      <c r="U182" s="2"/>
-      <c r="V182" s="2"/>
-    </row>
-    <row r="183" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="183" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A183" s="2"/>
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
@@ -6445,10 +6072,8 @@
       <c r="R183" s="2"/>
       <c r="S183" s="2"/>
       <c r="T183" s="2"/>
-      <c r="U183" s="2"/>
-      <c r="V183" s="2"/>
-    </row>
-    <row r="184" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="184" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A184" s="2"/>
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
@@ -6469,10 +6094,8 @@
       <c r="R184" s="2"/>
       <c r="S184" s="2"/>
       <c r="T184" s="2"/>
-      <c r="U184" s="2"/>
-      <c r="V184" s="2"/>
-    </row>
-    <row r="185" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="185" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A185" s="2"/>
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
@@ -6493,10 +6116,8 @@
       <c r="R185" s="2"/>
       <c r="S185" s="2"/>
       <c r="T185" s="2"/>
-      <c r="U185" s="2"/>
-      <c r="V185" s="2"/>
-    </row>
-    <row r="186" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="186" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A186" s="2"/>
       <c r="B186" s="2"/>
       <c r="C186" s="2"/>
@@ -6517,10 +6138,8 @@
       <c r="R186" s="2"/>
       <c r="S186" s="2"/>
       <c r="T186" s="2"/>
-      <c r="U186" s="2"/>
-      <c r="V186" s="2"/>
-    </row>
-    <row r="187" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="187" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A187" s="2"/>
       <c r="B187" s="2"/>
       <c r="C187" s="2"/>
@@ -6541,10 +6160,8 @@
       <c r="R187" s="2"/>
       <c r="S187" s="2"/>
       <c r="T187" s="2"/>
-      <c r="U187" s="2"/>
-      <c r="V187" s="2"/>
-    </row>
-    <row r="188" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="188" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A188" s="2"/>
       <c r="B188" s="2"/>
       <c r="C188" s="2"/>
@@ -6565,10 +6182,8 @@
       <c r="R188" s="2"/>
       <c r="S188" s="2"/>
       <c r="T188" s="2"/>
-      <c r="U188" s="2"/>
-      <c r="V188" s="2"/>
-    </row>
-    <row r="189" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="189" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A189" s="2"/>
       <c r="B189" s="2"/>
       <c r="C189" s="2"/>
@@ -6589,10 +6204,8 @@
       <c r="R189" s="2"/>
       <c r="S189" s="2"/>
       <c r="T189" s="2"/>
-      <c r="U189" s="2"/>
-      <c r="V189" s="2"/>
-    </row>
-    <row r="190" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="190" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A190" s="2"/>
       <c r="B190" s="2"/>
       <c r="C190" s="2"/>
@@ -6613,10 +6226,8 @@
       <c r="R190" s="2"/>
       <c r="S190" s="2"/>
       <c r="T190" s="2"/>
-      <c r="U190" s="2"/>
-      <c r="V190" s="2"/>
-    </row>
-    <row r="191" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="191" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A191" s="2"/>
       <c r="B191" s="2"/>
       <c r="C191" s="2"/>
@@ -6637,10 +6248,8 @@
       <c r="R191" s="2"/>
       <c r="S191" s="2"/>
       <c r="T191" s="2"/>
-      <c r="U191" s="2"/>
-      <c r="V191" s="2"/>
-    </row>
-    <row r="192" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="192" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A192" s="2"/>
       <c r="B192" s="2"/>
       <c r="C192" s="2"/>
@@ -6661,10 +6270,8 @@
       <c r="R192" s="2"/>
       <c r="S192" s="2"/>
       <c r="T192" s="2"/>
-      <c r="U192" s="2"/>
-      <c r="V192" s="2"/>
-    </row>
-    <row r="193" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="193" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A193" s="2"/>
       <c r="B193" s="2"/>
       <c r="C193" s="2"/>
@@ -6685,10 +6292,8 @@
       <c r="R193" s="2"/>
       <c r="S193" s="2"/>
       <c r="T193" s="2"/>
-      <c r="U193" s="2"/>
-      <c r="V193" s="2"/>
-    </row>
-    <row r="194" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="194" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A194" s="2"/>
       <c r="B194" s="2"/>
       <c r="C194" s="2"/>
@@ -6709,10 +6314,8 @@
       <c r="R194" s="2"/>
       <c r="S194" s="2"/>
       <c r="T194" s="2"/>
-      <c r="U194" s="2"/>
-      <c r="V194" s="2"/>
-    </row>
-    <row r="195" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="195" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A195" s="2"/>
       <c r="B195" s="2"/>
       <c r="C195" s="2"/>
@@ -6733,10 +6336,8 @@
       <c r="R195" s="2"/>
       <c r="S195" s="2"/>
       <c r="T195" s="2"/>
-      <c r="U195" s="2"/>
-      <c r="V195" s="2"/>
-    </row>
-    <row r="196" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="196" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A196" s="2"/>
       <c r="B196" s="2"/>
       <c r="C196" s="2"/>
@@ -6757,10 +6358,8 @@
       <c r="R196" s="2"/>
       <c r="S196" s="2"/>
       <c r="T196" s="2"/>
-      <c r="U196" s="2"/>
-      <c r="V196" s="2"/>
-    </row>
-    <row r="197" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="197" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A197" s="2"/>
       <c r="B197" s="2"/>
       <c r="C197" s="2"/>
@@ -6781,10 +6380,8 @@
       <c r="R197" s="2"/>
       <c r="S197" s="2"/>
       <c r="T197" s="2"/>
-      <c r="U197" s="2"/>
-      <c r="V197" s="2"/>
-    </row>
-    <row r="198" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="198" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A198" s="2"/>
       <c r="B198" s="2"/>
       <c r="C198" s="2"/>
@@ -6805,10 +6402,8 @@
       <c r="R198" s="2"/>
       <c r="S198" s="2"/>
       <c r="T198" s="2"/>
-      <c r="U198" s="2"/>
-      <c r="V198" s="2"/>
-    </row>
-    <row r="199" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="199" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A199" s="2"/>
       <c r="B199" s="2"/>
       <c r="C199" s="2"/>
@@ -6829,10 +6424,8 @@
       <c r="R199" s="2"/>
       <c r="S199" s="2"/>
       <c r="T199" s="2"/>
-      <c r="U199" s="2"/>
-      <c r="V199" s="2"/>
-    </row>
-    <row r="200" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="200" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A200" s="2"/>
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
@@ -6853,10 +6446,8 @@
       <c r="R200" s="2"/>
       <c r="S200" s="2"/>
       <c r="T200" s="2"/>
-      <c r="U200" s="2"/>
-      <c r="V200" s="2"/>
-    </row>
-    <row r="201" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="201" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A201" s="2"/>
       <c r="B201" s="2"/>
       <c r="C201" s="2"/>
@@ -6877,10 +6468,8 @@
       <c r="R201" s="2"/>
       <c r="S201" s="2"/>
       <c r="T201" s="2"/>
-      <c r="U201" s="2"/>
-      <c r="V201" s="2"/>
-    </row>
-    <row r="202" spans="1:22" x14ac:dyDescent="0.2">
+    </row>
+    <row r="202" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A202" s="2"/>
       <c r="B202" s="2"/>
       <c r="C202" s="2"/>
@@ -6901,44 +6490,42 @@
       <c r="R202" s="2"/>
       <c r="S202" s="2"/>
       <c r="T202" s="2"/>
-      <c r="U202" s="2"/>
-      <c r="V202" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="BTexII7owVy7UQbHfXi/pyJQyZY+TVM2NUjbJHtKkRwH9qU3D0asKSbCPlNE3BE//D65VD7VqTSzNJRUsWzKQw==" saltValue="9Bv0Uc7e1ZSaTefnMGuLyA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="11">
-    <mergeCell ref="T1:V1"/>
-    <mergeCell ref="R1:S1"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="R1:T1"/>
+    <mergeCell ref="P1:Q1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="E1:E2"/>
-    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="L1:N1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="D1:D2"/>
-    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="O1:O2"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E2 F2 H2 J2 L2 N2 Q1:Q2" xr:uid="{CF79E0B9-452F-42D7-82F9-4325C7CCE12E}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E2 F2 H2 I2 K2 L2 O1:O2" xr:uid="{CF79E0B9-452F-42D7-82F9-4325C7CCE12E}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
-    <dataValidation type="custom" sqref="P2" xr:uid="{746A974C-37B7-4392-8C1F-3624962D83AA}">
+    <dataValidation type="custom" sqref="N2" xr:uid="{746A974C-37B7-4392-8C1F-3624962D83AA}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="E1:E2" r:id="rId1" location="samplingMethodsForSamplingCollection" display="SAMPLING_METHOD" xr:uid="{863AF79D-449A-4B35-AC8D-9C415D8A32B9}"/>
     <hyperlink ref="H2" r:id="rId2" location="lengthMeasurementTools" xr:uid="{776CD30A-4D78-4230-9891-093ADBA1D96D}"/>
-    <hyperlink ref="L2" r:id="rId3" location="lengthMeasurementTools" xr:uid="{3DE19339-45B9-47B8-B5FB-D4012AD9C532}"/>
+    <hyperlink ref="K2" r:id="rId3" location="lengthMeasurementTools" xr:uid="{3DE19339-45B9-47B8-B5FB-D4012AD9C532}"/>
     <hyperlink ref="F2" r:id="rId4" location="lengthMeasurementTypes" xr:uid="{4F273766-A7DB-428C-A222-09DB4E6495A6}"/>
-    <hyperlink ref="J2" r:id="rId5" location="lengthMeasurementTypes" xr:uid="{50D5D995-3D3B-46CA-9856-C3BF09F867B6}"/>
-    <hyperlink ref="N2" r:id="rId6" location="fishProcessingTypes" xr:uid="{4C80F85B-DC5E-4379-AEDD-32355F2C04AE}"/>
-    <hyperlink ref="Q1:Q2" r:id="rId7" location="sex" display="SEX" xr:uid="{06582CBC-0354-4030-B121-DACE171DCC1B}"/>
-    <hyperlink ref="P2" r:id="rId8" location="weightMeasurementTools" xr:uid="{074E1E59-D343-4222-8E1C-310625164A04}"/>
-    <hyperlink ref="S2" r:id="rId9" location="Maturity_Stages" xr:uid="{E5D44B35-6082-4003-9C14-F412F3AFBAD6}"/>
-    <hyperlink ref="T2" r:id="rId10" location="samplingMethodsForSamplingCollection" xr:uid="{9F653EC4-D647-4197-B661-7CCACA627208}"/>
-    <hyperlink ref="U2" r:id="rId11" location="fishStorageTypes" xr:uid="{AA058992-D2B7-40CE-B6C6-3E8AA47DE46F}"/>
+    <hyperlink ref="I2" r:id="rId5" location="lengthMeasurementTypes" xr:uid="{50D5D995-3D3B-46CA-9856-C3BF09F867B6}"/>
+    <hyperlink ref="L2" r:id="rId6" location="fishProcessingTypes" xr:uid="{4C80F85B-DC5E-4379-AEDD-32355F2C04AE}"/>
+    <hyperlink ref="O1:O2" r:id="rId7" location="sex" display="SEX" xr:uid="{06582CBC-0354-4030-B121-DACE171DCC1B}"/>
+    <hyperlink ref="N2" r:id="rId8" location="weightMeasurementTools" xr:uid="{074E1E59-D343-4222-8E1C-310625164A04}"/>
+    <hyperlink ref="Q2" r:id="rId9" location="Maturity_Stages" xr:uid="{E5D44B35-6082-4003-9C14-F412F3AFBAD6}"/>
+    <hyperlink ref="R2" r:id="rId10" location="samplingMethodsForSamplingCollection" xr:uid="{9F653EC4-D647-4197-B661-7CCACA627208}"/>
+    <hyperlink ref="S2" r:id="rId11" location="fishStorageTypes" xr:uid="{AA058992-D2B7-40CE-B6C6-3E8AA47DE46F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6966,31 +6553,31 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="109" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="109" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="109" t="s">
+      <c r="C1" s="109" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="D1" s="109" t="s">
         <v>60</v>
       </c>
-      <c r="D1" s="109" t="s">
-        <v>61</v>
+      <c r="E1" s="93" t="s">
+        <v>170</v>
       </c>
-      <c r="E1" s="93" t="s">
+      <c r="F1" s="93" t="s">
         <v>171</v>
       </c>
-      <c r="F1" s="93" t="s">
+      <c r="G1" s="93" t="s">
         <v>172</v>
-      </c>
-      <c r="G1" s="93" t="s">
-        <v>173</v>
       </c>
       <c r="H1" s="111" t="s">
         <v>42</v>
       </c>
       <c r="I1" s="94" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J1" s="111" t="s">
         <v>43</v>
@@ -9663,16 +9250,16 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="46" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="46" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="C1" s="46" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="D1" s="46" t="s">
         <v>60</v>
-      </c>
-      <c r="D1" s="46" t="s">
-        <v>61</v>
       </c>
       <c r="E1" s="39" t="s">
         <v>40</v>
@@ -9684,19 +9271,19 @@
         <v>19</v>
       </c>
       <c r="H1" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="I1" s="39" t="s">
         <v>191</v>
       </c>
-      <c r="I1" s="39" t="s">
-        <v>192</v>
+      <c r="J1" s="39" t="s">
+        <v>174</v>
       </c>
-      <c r="J1" s="39" t="s">
+      <c r="K1" s="39" t="s">
         <v>175</v>
       </c>
-      <c r="K1" s="39" t="s">
-        <v>176</v>
-      </c>
       <c r="L1" s="49" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -12531,10 +12118,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="34" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C1" s="34" t="s">
         <v>0</v>
@@ -12543,10 +12130,10 @@
         <v>1</v>
       </c>
       <c r="E1" s="30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F1" s="34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -14196,14 +13783,14 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="62" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="62" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C1" s="62"/>
       <c r="D1" s="62" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E1" s="62"/>
       <c r="F1" s="62"/>
@@ -14215,7 +13802,7 @@
       <c r="L1" s="62"/>
       <c r="M1" s="62"/>
       <c r="N1" s="62" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O1" s="62"/>
       <c r="P1" s="62"/>
@@ -14234,14 +13821,14 @@
       <c r="B2" s="62"/>
       <c r="C2" s="62"/>
       <c r="D2" s="65" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E2" s="66"/>
       <c r="F2" s="66"/>
       <c r="G2" s="66"/>
       <c r="H2" s="71"/>
       <c r="I2" s="65" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J2" s="66"/>
       <c r="K2" s="66"/>
@@ -14265,40 +13852,40 @@
       <c r="B3" s="62"/>
       <c r="C3" s="62"/>
       <c r="D3" s="67" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E3" s="68"/>
       <c r="F3" s="63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G3" s="64"/>
       <c r="H3" s="69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I3" s="67" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J3" s="68"/>
       <c r="K3" s="63" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L3" s="64"/>
       <c r="M3" s="69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="N3" s="62" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O3" s="62"/>
       <c r="P3" s="62" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q3" s="62"/>
       <c r="R3" s="62"/>
       <c r="S3" s="62"/>
       <c r="T3" s="62"/>
       <c r="U3" s="72" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="V3" s="73"/>
       <c r="W3" s="73"/>
@@ -14307,13 +13894,13 @@
     <row r="4" spans="1:25" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="62"/>
       <c r="B4" s="31" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" s="34" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E4" s="30" t="s">
         <v>4</v>
@@ -14326,7 +13913,7 @@
       </c>
       <c r="H4" s="70"/>
       <c r="I4" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J4" s="30" t="s">
         <v>4</v>
@@ -14360,16 +13947,16 @@
         <v>10</v>
       </c>
       <c r="U4" s="30" t="s">
+        <v>105</v>
+      </c>
+      <c r="V4" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="V4" s="30" t="s">
+      <c r="W4" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="W4" s="30" t="s">
+      <c r="X4" s="30" t="s">
         <v>108</v>
-      </c>
-      <c r="X4" s="30" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.2">
@@ -14663,7 +14250,7 @@
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -19615,7 +19202,7 @@
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="76" t="s">
         <v>17</v>
@@ -19630,13 +19217,13 @@
       <c r="H1" s="89"/>
       <c r="I1" s="90"/>
       <c r="J1" s="93" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K1" s="96" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L1" s="76" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M1" s="77"/>
       <c r="N1" s="77"/>
@@ -19649,7 +19236,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="86" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D2" s="62" t="s">
         <v>2</v>
@@ -19661,22 +19248,22 @@
         <v>14</v>
       </c>
       <c r="G2" s="83" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H2" s="84" t="s">
         <v>4</v>
       </c>
       <c r="I2" s="91" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J2" s="94"/>
       <c r="K2" s="97"/>
       <c r="L2" s="79" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M2" s="79"/>
       <c r="N2" s="79" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O2" s="79"/>
       <c r="P2" s="80" t="s">
@@ -19699,13 +19286,13 @@
         <v>3</v>
       </c>
       <c r="M3" s="35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="N3" s="31" t="s">
         <v>3</v>
       </c>
       <c r="O3" s="35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P3" s="80"/>
     </row>
@@ -23374,17 +22961,17 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="79" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C1" s="79"/>
       <c r="D1" s="79"/>
       <c r="E1" s="79"/>
       <c r="F1" s="79"/>
       <c r="G1" s="79" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H1" s="79"/>
       <c r="I1" s="79"/>
@@ -23394,28 +22981,28 @@
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="75"/>
       <c r="B2" s="65" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2" s="66"/>
       <c r="D2" s="66"/>
       <c r="E2" s="66"/>
       <c r="F2" s="69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G2" s="65" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H2" s="66"/>
       <c r="I2" s="66"/>
       <c r="J2" s="71"/>
       <c r="K2" s="69" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="70"/>
       <c r="B3" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C3" s="30" t="s">
         <v>4</v>
@@ -23428,7 +23015,7 @@
       </c>
       <c r="F3" s="70"/>
       <c r="G3" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H3" s="30" t="s">
         <v>4</v>
@@ -26116,10 +25703,10 @@
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="72" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C1" s="73"/>
       <c r="D1" s="73"/>
@@ -26140,7 +25727,7 @@
       <c r="S1" s="73"/>
       <c r="T1" s="74"/>
       <c r="U1" s="72" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="V1" s="73"/>
       <c r="W1" s="73"/>
@@ -26155,7 +25742,7 @@
       <c r="AF1" s="73"/>
       <c r="AG1" s="74"/>
       <c r="AH1" s="72" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="AI1" s="73"/>
       <c r="AJ1" s="73"/>
@@ -26168,35 +25755,35 @@
     <row r="2" spans="1:41" x14ac:dyDescent="0.2">
       <c r="A2" s="75"/>
       <c r="B2" s="81" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="100" t="s">
         <v>181</v>
       </c>
-      <c r="C2" s="100" t="s">
-        <v>182</v>
-      </c>
       <c r="D2" s="93" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E2" s="99" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F2" s="99"/>
       <c r="G2" s="99"/>
       <c r="H2" s="99" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="I2" s="99"/>
       <c r="J2" s="99"/>
       <c r="K2" s="101" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L2" s="87" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M2" s="87"/>
       <c r="N2" s="87"/>
       <c r="O2" s="87"/>
       <c r="P2" s="99" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Q2" s="99"/>
       <c r="R2" s="99"/>
@@ -26205,7 +25792,7 @@
       </c>
       <c r="T2" s="87"/>
       <c r="U2" s="112" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="V2" s="112" t="s">
         <v>23</v>
@@ -26244,19 +25831,19 @@
         <v>33</v>
       </c>
       <c r="AH2" s="87" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AI2" s="87"/>
       <c r="AJ2" s="87" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="AK2" s="87"/>
       <c r="AL2" s="87" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="AM2" s="87"/>
       <c r="AN2" s="87" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AO2" s="87"/>
     </row>
@@ -26272,7 +25859,7 @@
         <v>21</v>
       </c>
       <c r="G3" s="47" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H3" s="47" t="s">
         <v>20</v>
@@ -26281,35 +25868,35 @@
         <v>21</v>
       </c>
       <c r="J3" s="47" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K3" s="102"/>
       <c r="L3" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="M3" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="M3" s="30" t="s">
+      <c r="N3" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="N3" s="30" t="s">
+      <c r="O3" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="O3" s="30" t="s">
-        <v>122</v>
+      <c r="P3" s="33" t="s">
+        <v>124</v>
       </c>
-      <c r="P3" s="33" t="s">
+      <c r="Q3" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="Q3" s="33" t="s">
+      <c r="R3" s="33" t="s">
         <v>126</v>
-      </c>
-      <c r="R3" s="33" t="s">
-        <v>127</v>
       </c>
       <c r="S3" s="34" t="s">
         <v>18</v>
       </c>
       <c r="T3" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="U3" s="112"/>
       <c r="V3" s="112"/>
@@ -26325,28 +25912,28 @@
       <c r="AF3" s="112"/>
       <c r="AG3" s="112"/>
       <c r="AH3" s="41" t="s">
+        <v>129</v>
+      </c>
+      <c r="AI3" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="AI3" s="33" t="s">
+      <c r="AJ3" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="AJ3" s="33" t="s">
+      <c r="AK3" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="AK3" s="33" t="s">
+      <c r="AL3" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="AL3" s="33" t="s">
+      <c r="AM3" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="AM3" s="33" t="s">
+      <c r="AN3" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="AN3" s="33" t="s">
+      <c r="AO3" s="33" t="s">
         <v>136</v>
-      </c>
-      <c r="AO3" s="33" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.2">
@@ -35040,14 +34627,14 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" s="72" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C1" s="74"/>
       <c r="D1" s="72" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E1" s="73"/>
       <c r="F1" s="73"/>
@@ -35061,25 +34648,25 @@
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="75"/>
       <c r="B2" s="113" t="s">
+        <v>61</v>
+      </c>
+      <c r="C2" s="113" t="s">
         <v>62</v>
       </c>
-      <c r="C2" s="113" t="s">
+      <c r="D2" s="87" t="s">
         <v>63</v>
-      </c>
-      <c r="D2" s="87" t="s">
-        <v>64</v>
       </c>
       <c r="E2" s="87"/>
       <c r="F2" s="87"/>
       <c r="G2" s="87"/>
       <c r="H2" s="87" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I2" s="87"/>
       <c r="J2" s="87"/>
       <c r="K2" s="87"/>
       <c r="L2" s="87" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -35087,19 +34674,19 @@
       <c r="B3" s="113"/>
       <c r="C3" s="113"/>
       <c r="D3" s="87" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E3" s="87"/>
       <c r="F3" s="87" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G3" s="87"/>
       <c r="H3" s="87" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I3" s="87"/>
       <c r="J3" s="87" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K3" s="87"/>
       <c r="L3" s="87"/>
@@ -35112,28 +34699,28 @@
         <v>18</v>
       </c>
       <c r="E4" s="45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F4" s="45" t="s">
         <v>18</v>
       </c>
       <c r="G4" s="45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H4" s="45" t="s">
         <v>18</v>
       </c>
       <c r="I4" s="45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="J4" s="45" t="s">
         <v>18</v>
       </c>
       <c r="K4" s="45" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L4" s="34" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -37988,46 +37575,46 @@
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="69" t="s">
-        <v>59</v>
-      </c>
       <c r="C1" s="65" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D1" s="66"/>
       <c r="E1" s="71"/>
       <c r="F1" s="100" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G1" s="103"/>
       <c r="H1" s="103"/>
       <c r="I1" s="103"/>
       <c r="J1" s="96" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="K1" s="105" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L1" s="87" t="s">
+        <v>64</v>
+      </c>
+      <c r="M1" s="87" t="s">
         <v>65</v>
       </c>
-      <c r="M1" s="87" t="s">
+      <c r="N1" s="87" t="s">
         <v>66</v>
-      </c>
-      <c r="N1" s="87" t="s">
-        <v>67</v>
       </c>
       <c r="O1" s="72"/>
       <c r="P1" s="69" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q1" s="74" t="s">
         <v>68</v>
       </c>
-      <c r="Q1" s="74" t="s">
-        <v>69</v>
-      </c>
       <c r="R1" s="87" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="S1" s="87"/>
       <c r="T1" s="87"/>
@@ -38038,10 +37625,10 @@
       <c r="A2" s="75"/>
       <c r="B2" s="75"/>
       <c r="C2" s="106" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D2" s="65" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E2" s="71"/>
       <c r="F2" s="67"/>
@@ -38057,14 +37644,14 @@
       <c r="P2" s="75"/>
       <c r="Q2" s="74"/>
       <c r="R2" s="99" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S2" s="87" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="T2" s="87"/>
       <c r="U2" s="87" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="V2" s="87"/>
     </row>
@@ -38079,41 +37666,41 @@
         <v>1</v>
       </c>
       <c r="F3" s="30" t="s">
+        <v>150</v>
+      </c>
+      <c r="G3" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="G3" s="30" t="s">
+      <c r="H3" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="I3" s="43" t="s">
         <v>153</v>
-      </c>
-      <c r="I3" s="43" t="s">
-        <v>154</v>
       </c>
       <c r="J3" s="98"/>
       <c r="K3" s="105"/>
       <c r="L3" s="87"/>
       <c r="M3" s="87"/>
       <c r="N3" s="36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O3" s="42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P3" s="70"/>
       <c r="Q3" s="74"/>
       <c r="R3" s="99"/>
       <c r="S3" s="114" t="s">
+        <v>72</v>
+      </c>
+      <c r="T3" s="114" t="s">
         <v>73</v>
       </c>
-      <c r="T3" s="114" t="s">
-        <v>74</v>
-      </c>
       <c r="U3" s="33" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="V3" s="33" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.2">
@@ -42977,22 +42564,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="31" t="s">
-        <v>59</v>
-      </c>
       <c r="C1" s="115" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E1" s="31" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F1" s="115" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -44633,26 +44220,26 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="69" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="69" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="69" t="s">
+      <c r="C1" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="C1" s="69" t="s">
-        <v>60</v>
-      </c>
       <c r="D1" s="96" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E1" s="107" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F1" s="108"/>
       <c r="G1" s="96" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H1" s="69" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I1" s="65" t="s">
         <v>35</v>
@@ -44669,18 +44256,18 @@
         <v>19</v>
       </c>
       <c r="F2" s="38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G2" s="98"/>
       <c r="H2" s="70"/>
       <c r="I2" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="J2" s="50" t="s">
         <v>36</v>
       </c>
       <c r="K2" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
adding logical responses code list to specimen - brought onboard and revival fields
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BF7B744-D3EA-9342-9A98-97FC8850D4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E655CDB6-0B65-AF48-A000-1E7FBFA54934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="c5/ou8Cml7ZkaDU47Tuu3WsAbYP19DC42wRzPBn3vsHWJE2MFn5j3m9vhk0UNMu/icNe5bym2Fttv6xJI1ZSAw==" workbookSaltValue="pG4NehU6lkQVWVHx3qNlvg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16360" tabRatio="879" firstSheet="1" activeTab="9" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16420" tabRatio="879" firstSheet="9" activeTab="10" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -991,7 +991,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
@@ -1327,6 +1327,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -6573,13 +6579,13 @@
       <c r="G1" s="93" t="s">
         <v>172</v>
       </c>
-      <c r="H1" s="111" t="s">
+      <c r="H1" s="116" t="s">
         <v>42</v>
       </c>
       <c r="I1" s="94" t="s">
         <v>173</v>
       </c>
-      <c r="J1" s="111" t="s">
+      <c r="J1" s="116" t="s">
         <v>43</v>
       </c>
       <c r="K1" s="111" t="s">
@@ -6594,9 +6600,9 @@
       <c r="E2" s="95"/>
       <c r="F2" s="95"/>
       <c r="G2" s="95"/>
-      <c r="H2" s="82"/>
+      <c r="H2" s="117"/>
       <c r="I2" s="95"/>
-      <c r="J2" s="82"/>
+      <c r="J2" s="117"/>
       <c r="K2" s="82"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -9200,7 +9206,7 @@
       <c r="K202" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="/i8ttRawHFE0bDsLHk0X3DAZnREwIVUNut+wCnlTtUXkhO/z6EY5v2kRXopEus0UfjIHrMc29E3tZKRlwPN6dQ==" saltValue="ZTcyu138evLLcD0f3mUgnw==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="UEOkJqql+6bXjzeDjXVTayAmYnh9n1oqPSFnV6umLOYr9lZtqV9rKz85k3fGQuh6t2Yr3DiOx//LRdvP061mOQ==" saltValue="+R1cJAk8uUHACXVc/8Bf3w==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <mergeCells count="11">
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="I1:I2"/>
@@ -9226,9 +9232,11 @@
     <hyperlink ref="F1" r:id="rId4" location="individualConditions" display="CONDITION_AT_RELEASE_CODE" xr:uid="{312D6457-0D67-4610-B478-F5AE649B98F6}"/>
     <hyperlink ref="E1:E2" r:id="rId5" location="individualConditions" display="CONDITION_AT_CAPTURE" xr:uid="{F4906E56-6A88-4C64-867C-2ABD778A70BA}"/>
     <hyperlink ref="F1:F2" r:id="rId6" location="individualConditions" display="CONDITION_AT_RELEASE" xr:uid="{EFA1D569-0D47-49ED-B0FE-53D3A24E5072}"/>
+    <hyperlink ref="H1:H2" r:id="rId7" location="logicalResponses" display="BROUGHT_ONBOARD" xr:uid="{BE2D5C4E-F649-A249-B9E9-4C28A175E0FB}"/>
+    <hyperlink ref="J1:J2" r:id="rId8" location="logicalResponses" display="REVIVAL" xr:uid="{C7306B6C-F527-5849-8C5B-733F17EACDC6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
logical response code lists added to tag details: release and recovery
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ros/Form-ROS-PS.xlsx
+++ b/form_reporting_templates/ros/Form-ROS-PS.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_reporting_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E655CDB6-0B65-AF48-A000-1E7FBFA54934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF65BCDF-65DF-1B4E-B7A8-E00BD04FB54F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="c5/ou8Cml7ZkaDU47Tuu3WsAbYP19DC42wRzPBn3vsHWJE2MFn5j3m9vhk0UNMu/icNe5bym2Fttv6xJI1ZSAw==" workbookSaltValue="pG4NehU6lkQVWVHx3qNlvg==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16420" tabRatio="879" firstSheet="9" activeTab="10" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
+    <workbookView xWindow="160" yWindow="900" windowWidth="29080" windowHeight="16420" tabRatio="879" firstSheet="9" activeTab="11" xr2:uid="{EFC17563-B14E-425F-8BEA-A9EB7F2C43CD}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="26" r:id="rId1"/>
@@ -9269,10 +9269,10 @@
       <c r="D1" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="39" t="s">
+      <c r="E1" s="114" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="39" t="s">
+      <c r="F1" s="114" t="s">
         <v>41</v>
       </c>
       <c r="G1" s="33" t="s">
@@ -12095,7 +12095,7 @@
       <c r="L201" s="6"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="atCsfaQ/Wqa05oY0/VI6TFi+I2NXWNTJgSm76H37XWGla1PXU95wuw4Y7lxV3gUUgepEXdCeLWyl2wtd/jFNBQ==" saltValue="bBGMR4jLd0WwJNjJRc35BQ==" spinCount="100000" sheet="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="QMw2cG8bGvhh0Fd8tMDI22dYVyFI/+1OdAQh7QlavhKJrDyuSu6VqVJ6uqpP8ZzZ8VOBXTcz3nOpUwlBJ2ge4w==" saltValue="VzeJkKzahBCc5aLAXJwkGA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1" xr:uid="{4FDCD393-A02F-41DC-AAE5-5D41DD47867C}">
       <formula1>"&lt;0&gt;0"</formula1>
@@ -12103,6 +12103,8 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="G1" r:id="rId1" location="tagTypes" xr:uid="{ECAFC5F2-6FEB-4806-8763-D5FABB0EB5EB}"/>
+    <hyperlink ref="E1" r:id="rId2" location="logicalResponses" xr:uid="{4978B5C2-9384-0242-8D3E-118677427F5C}"/>
+    <hyperlink ref="F1" r:id="rId3" location="logicalResponses" xr:uid="{198380F3-20E3-D84F-90EB-5F522A6A7667}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>